<commit_message>
IC startingover image output raw
</commit_message>
<xml_diff>
--- a/ppm_output_handcalc.xlsx
+++ b/ppm_output_handcalc.xlsx
@@ -8,19 +8,58 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drirpy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EBEB36-C452-B74B-A6DD-191E3C6A1B7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438713BA-10E2-7841-86B8-724BCA30CCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPM" sheetId="1" r:id="rId1"/>
+    <sheet name="Information Content" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="PPM">PPM!$A$1:$M$5</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
   <si>
     <t>A</t>
   </si>
@@ -33,12 +72,27 @@
   <si>
     <t>T</t>
   </si>
+  <si>
+    <t>Metric: Information Content</t>
+  </si>
+  <si>
+    <t>H_after</t>
+  </si>
+  <si>
+    <t>P_XY</t>
+  </si>
+  <si>
+    <t>Result (H_before - H_after)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,13 +106,40 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -88,11 +169,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -114,16 +212,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>24423</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>73269</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>268654</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>364066</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>608298</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>47089</xdr:rowOff>
+      <xdr:rowOff>161063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -146,7 +244,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="700128" y="1196731"/>
+          <a:off x="268654" y="1310705"/>
           <a:ext cx="7772400" cy="3718691"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -448,7 +546,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1" s="1">
+      <c r="B1" s="8">
         <v>0</v>
       </c>
       <c r="C1" s="1">
@@ -653,4 +751,705 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C6B552-D222-D944-AA0C-60A0FCCF6FC4}">
+  <dimension ref="A1:T13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="9" width="5.5" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" customWidth="1"/>
+    <col min="11" max="11" width="8.1640625" customWidth="1"/>
+    <col min="12" max="12" width="7.5" customWidth="1"/>
+    <col min="13" max="13" width="6.1640625" customWidth="1"/>
+    <col min="15" max="15" width="4.1640625" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" customWidth="1"/>
+    <col min="20" max="20" width="12.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1">
+        <v>11</v>
+      </c>
+      <c r="P1" s="9">
+        <v>7</v>
+      </c>
+      <c r="Q1" s="9">
+        <v>2</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="5">
+        <v>0.38745151999999999</v>
+      </c>
+      <c r="D2">
+        <f xml:space="preserve"> 0.945815271</f>
+        <v>0.94581527099999996</v>
+      </c>
+      <c r="E2">
+        <v>0.60167079231986764</v>
+      </c>
+      <c r="F2">
+        <v>0.37505516144940576</v>
+      </c>
+      <c r="G2">
+        <v>0.59676075799999995</v>
+      </c>
+      <c r="H2">
+        <v>0.500655077</v>
+      </c>
+      <c r="I2">
+        <v>1.0382551289999999</v>
+      </c>
+      <c r="J2">
+        <v>0.46412009799999998</v>
+      </c>
+      <c r="K2">
+        <v>0.91279231299999997</v>
+      </c>
+      <c r="L2">
+        <v>0.60167079199999995</v>
+      </c>
+      <c r="M2" s="10">
+        <v>0.34988060900000001</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" cm="1">
+        <f t="array" ref="P2">INDEX(PPM!$B$2:$M$5, ROW(A1), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1.5625000100000001E-2</v>
+      </c>
+      <c r="Q2" cm="1">
+        <f t="array" ref="Q2">INDEX(PPM!$B$2:$M$5, ROW(B1), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="R2" s="5">
+        <f>AVERAGE(P2,Q2)</f>
+        <v>7.8125001000000013E-3</v>
+      </c>
+      <c r="S2">
+        <f xml:space="preserve"> R2*LOG(R2, 2)</f>
+        <v>-5.4687500555730503E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" cm="1">
+        <f t="array" ref="B3">INDEX($B$2:$M$13, COLUMN(A2), ROW(A2))</f>
+        <v>0.38745151999999999</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3">
+        <v>0.80600252400000005</v>
+      </c>
+      <c r="E3">
+        <v>0.944073524</v>
+      </c>
+      <c r="F3">
+        <v>0.94300772600000005</v>
+      </c>
+      <c r="G3" s="5">
+        <v>0.43011038600000001</v>
+      </c>
+      <c r="H3">
+        <v>1.7740252299999999</v>
+      </c>
+      <c r="I3">
+        <v>0.41379671899999998</v>
+      </c>
+      <c r="J3">
+        <v>1.7338225279999999</v>
+      </c>
+      <c r="K3">
+        <v>0.831354963</v>
+      </c>
+      <c r="L3">
+        <v>0.944073524</v>
+      </c>
+      <c r="M3">
+        <v>1.300679519</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" cm="1">
+        <f t="array" ref="P3">INDEX(PPM!$B$2:$M$5, ROW(A2), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.25000000010000001</v>
+      </c>
+      <c r="Q3" cm="1">
+        <f t="array" ref="Q3">INDEX(PPM!$B$2:$M$5, ROW(B2), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.98437500010000001</v>
+      </c>
+      <c r="R3" s="5">
+        <f t="shared" ref="R3:R5" si="0">AVERAGE(P3,Q3)</f>
+        <v>0.61718750010000001</v>
+      </c>
+      <c r="S3">
+        <f t="shared" ref="S3:S5" si="1" xml:space="preserve"> R3*LOG(R3, 2)</f>
+        <v>-0.42969781940979673</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" cm="1">
+        <f t="array" ref="B4">INDEX($B$2:$M$13, COLUMN(A3), ROW(A3))</f>
+        <v>0.94581527099999996</v>
+      </c>
+      <c r="C4" s="5" cm="1">
+        <f t="array" ref="C4">INDEX($B$2:$M$13, COLUMN(B3), ROW(B3))</f>
+        <v>0.80600252400000005</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4">
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="F4">
+        <v>0.71751021720520058</v>
+      </c>
+      <c r="G4">
+        <v>0.52122605644552022</v>
+      </c>
+      <c r="H4">
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="I4">
+        <v>0.984975614485744</v>
+      </c>
+      <c r="J4">
+        <v>0.88388492366776417</v>
+      </c>
+      <c r="K4">
+        <v>1.8682599204038386</v>
+      </c>
+      <c r="L4">
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="M4">
+        <v>0.97954808599999998</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P4" cm="1">
+        <f t="array" ref="P4">INDEX(PPM!$B$2:$M$5, ROW(A3), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.73437500010000001</v>
+      </c>
+      <c r="Q4" cm="1">
+        <f t="array" ref="Q4">INDEX(PPM!$B$2:$M$5, ROW(B3), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1.5625000100000001E-2</v>
+      </c>
+      <c r="R4" s="5">
+        <f t="shared" si="0"/>
+        <v>0.37500000010000001</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="1"/>
+        <v>-0.53063906222680068</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" cm="1">
+        <f t="array" ref="B5">INDEX($B$2:$M$13, COLUMN(A4), ROW(A4))</f>
+        <v>0.60167079231986764</v>
+      </c>
+      <c r="C5" s="5" cm="1">
+        <f t="array" ref="C5">INDEX($B$2:$M$13, COLUMN(B4), ROW(B4))</f>
+        <v>0.944073524</v>
+      </c>
+      <c r="D5" s="5" cm="1">
+        <f t="array" ref="D5">INDEX($B$2:$M$13, COLUMN(C4), ROW(C4))</f>
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5">
+        <v>1.7270291352821832</v>
+      </c>
+      <c r="G5">
+        <v>0.42898139485067821</v>
+      </c>
+      <c r="H5">
+        <v>0.99999999344468282</v>
+      </c>
+      <c r="I5">
+        <v>0.59780924559747062</v>
+      </c>
+      <c r="J5">
+        <v>1.000176111</v>
+      </c>
+      <c r="K5">
+        <v>1.0001761108457747</v>
+      </c>
+      <c r="L5">
+        <v>1.9999999901784853</v>
+      </c>
+      <c r="M5">
+        <v>0.60721985043626692</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P5" cm="1">
+        <f t="array" ref="P5">INDEX(PPM!$B$2:$M$5, ROW(A4), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="Q5" cm="1">
+        <f t="array" ref="Q5">INDEX(PPM!$B$2:$M$5, ROW(B4), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="R5" s="5">
+        <f t="shared" si="0"/>
+        <v>1E-10</v>
+      </c>
+      <c r="S5">
+        <f t="shared" si="1"/>
+        <v>-3.3219280948873626E-9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" cm="1">
+        <f t="array" ref="B6">INDEX($B$2:$M$13, COLUMN(A5), ROW(A5))</f>
+        <v>0.37505516144940576</v>
+      </c>
+      <c r="C6" s="5" cm="1">
+        <f t="array" ref="C6">INDEX($B$2:$M$13, COLUMN(B5), ROW(B5))</f>
+        <v>0.94300772600000005</v>
+      </c>
+      <c r="D6" s="5" cm="1">
+        <f t="array" ref="D6">INDEX($B$2:$M$13, COLUMN(C5), ROW(C5))</f>
+        <v>0.71751021720520058</v>
+      </c>
+      <c r="E6" s="5" cm="1">
+        <f t="array" ref="E6">INDEX($B$2:$M$13, COLUMN(D5), ROW(D5))</f>
+        <v>1.7270291352821832</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6">
+        <v>0.31750411260070321</v>
+      </c>
+      <c r="H6">
+        <v>1.006349282</v>
+      </c>
+      <c r="I6">
+        <v>0.37227649099999999</v>
+      </c>
+      <c r="J6">
+        <v>1.0044072390000001</v>
+      </c>
+      <c r="K6">
+        <v>0.77464335699999998</v>
+      </c>
+      <c r="L6">
+        <v>1.727029135</v>
+      </c>
+      <c r="M6">
+        <v>0.59641437900000005</v>
+      </c>
+      <c r="R6">
+        <f xml:space="preserve"> SUM(R2:R5)</f>
+        <v>1.0000000004</v>
+      </c>
+      <c r="S6" s="3">
+        <f>-SUM(S2:S5)</f>
+        <v>1.015024385514256</v>
+      </c>
+      <c r="T6">
+        <f xml:space="preserve"> 2 - S6</f>
+        <v>0.984975614485744</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" cm="1">
+        <f t="array" ref="B7">INDEX($B$2:$M$13, COLUMN(A6), ROW(A6))</f>
+        <v>0.59676075799999995</v>
+      </c>
+      <c r="C7" s="5" cm="1">
+        <f t="array" ref="C7">INDEX($B$2:$M$13, COLUMN(B6), ROW(B6))</f>
+        <v>0.43011038600000001</v>
+      </c>
+      <c r="D7" s="5" cm="1">
+        <f t="array" ref="D7">INDEX($B$2:$M$13, COLUMN(C6), ROW(C6))</f>
+        <v>0.52122605644552022</v>
+      </c>
+      <c r="E7" s="5" cm="1">
+        <f t="array" ref="E7">INDEX($B$2:$M$13, COLUMN(D6), ROW(D6))</f>
+        <v>0.42898139485067821</v>
+      </c>
+      <c r="F7" s="5" cm="1">
+        <f t="array" ref="F7">INDEX($B$2:$M$13, COLUMN(E6), ROW(E6))</f>
+        <v>0.31750411260070321</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7">
+        <v>0.52851445699999999</v>
+      </c>
+      <c r="I7">
+        <v>0.62406583999999998</v>
+      </c>
+      <c r="J7">
+        <v>0.50116565400000002</v>
+      </c>
+      <c r="K7">
+        <v>0.50116565400000002</v>
+      </c>
+      <c r="L7">
+        <v>0.42898139499999999</v>
+      </c>
+      <c r="M7">
+        <v>0.29768254</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="5" cm="1">
+        <f t="array" ref="B8">INDEX($B$2:$M$13, COLUMN(A7), ROW(A7))</f>
+        <v>0.500655077</v>
+      </c>
+      <c r="C8" s="5" cm="1">
+        <f t="array" ref="C8">INDEX($B$2:$M$13, COLUMN(B7), ROW(B7))</f>
+        <v>1.7740252299999999</v>
+      </c>
+      <c r="D8" s="5" cm="1">
+        <f t="array" ref="D8">INDEX($B$2:$M$13, COLUMN(C7), ROW(C7))</f>
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="E8" s="5" cm="1">
+        <f t="array" ref="E8">INDEX($B$2:$M$13, COLUMN(D7), ROW(D7))</f>
+        <v>0.99999999344468282</v>
+      </c>
+      <c r="F8" s="5" cm="1">
+        <f t="array" ref="F8">INDEX($B$2:$M$13, COLUMN(E7), ROW(E7))</f>
+        <v>1.006349282</v>
+      </c>
+      <c r="G8" s="5" cm="1">
+        <f t="array" ref="G8">INDEX($B$2:$M$13, COLUMN(F7), ROW(F7))</f>
+        <v>0.52851445699999999</v>
+      </c>
+      <c r="H8" s="2"/>
+      <c r="I8">
+        <v>0.53957559300000002</v>
+      </c>
+      <c r="J8">
+        <v>1.9340855809999999</v>
+      </c>
+      <c r="K8">
+        <v>0.94194245899999995</v>
+      </c>
+      <c r="L8">
+        <v>0.99999999299999998</v>
+      </c>
+      <c r="M8">
+        <v>1.4787779750000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" cm="1">
+        <f t="array" ref="B9">INDEX($B$2:$M$13, COLUMN(A8), ROW(A8))</f>
+        <v>1.0382551289999999</v>
+      </c>
+      <c r="C9" s="5" cm="1">
+        <f t="array" ref="C9">INDEX($B$2:$M$13, COLUMN(B8), ROW(B8))</f>
+        <v>0.41379671899999998</v>
+      </c>
+      <c r="D9" s="5" cm="1">
+        <f t="array" ref="D9">INDEX($B$2:$M$13, COLUMN(C8), ROW(C8))</f>
+        <v>0.984975614485744</v>
+      </c>
+      <c r="E9" s="5" cm="1">
+        <f t="array" ref="E9">INDEX($B$2:$M$13, COLUMN(D8), ROW(D8))</f>
+        <v>0.59780924559747062</v>
+      </c>
+      <c r="F9" s="5" cm="1">
+        <f t="array" ref="F9">INDEX($B$2:$M$13, COLUMN(E8), ROW(E8))</f>
+        <v>0.37227649099999999</v>
+      </c>
+      <c r="G9" s="5" cm="1">
+        <f t="array" ref="G9">INDEX($B$2:$M$13, COLUMN(F8), ROW(F8))</f>
+        <v>0.62406583999999998</v>
+      </c>
+      <c r="H9" s="5" cm="1">
+        <f t="array" ref="H9">INDEX($B$2:$M$13, COLUMN(G8), ROW(G8))</f>
+        <v>0.53957559300000002</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9">
+        <v>0.49714305600000003</v>
+      </c>
+      <c r="K9">
+        <v>0.94581527099999996</v>
+      </c>
+      <c r="L9">
+        <v>0.59780924599999996</v>
+      </c>
+      <c r="M9">
+        <v>0.388801124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" cm="1">
+        <f t="array" ref="B10">INDEX($B$2:$M$13, COLUMN(A9), ROW(A9))</f>
+        <v>0.46412009799999998</v>
+      </c>
+      <c r="C10" s="5" cm="1">
+        <f t="array" ref="C10">INDEX($B$2:$M$13, COLUMN(B9), ROW(B9))</f>
+        <v>1.7338225279999999</v>
+      </c>
+      <c r="D10" s="5" cm="1">
+        <f t="array" ref="D10">INDEX($B$2:$M$13, COLUMN(C9), ROW(C9))</f>
+        <v>0.88388492366776417</v>
+      </c>
+      <c r="E10" s="5" cm="1">
+        <f t="array" ref="E10">INDEX($B$2:$M$13, COLUMN(D9), ROW(D9))</f>
+        <v>1.000176111</v>
+      </c>
+      <c r="F10" s="5" cm="1">
+        <f t="array" ref="F10">INDEX($B$2:$M$13, COLUMN(E9), ROW(E9))</f>
+        <v>1.0044072390000001</v>
+      </c>
+      <c r="G10" s="5" cm="1">
+        <f t="array" ref="G10">INDEX($B$2:$M$13, COLUMN(F9), ROW(F9))</f>
+        <v>0.50116565400000002</v>
+      </c>
+      <c r="H10" s="5" cm="1">
+        <f t="array" ref="H10">INDEX($B$2:$M$13, COLUMN(G9), ROW(G9))</f>
+        <v>1.9340855809999999</v>
+      </c>
+      <c r="I10" s="5" cm="1">
+        <f t="array" ref="I10">INDEX($B$2:$M$13, COLUMN(H9), ROW(H9))</f>
+        <v>0.49714305600000003</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="5">
+        <v>0.89950992100000005</v>
+      </c>
+      <c r="L10">
+        <v>1.000176111</v>
+      </c>
+      <c r="M10">
+        <v>1.414274295</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" cm="1">
+        <f t="array" ref="B11">INDEX($B$2:$M$13, COLUMN(A10), ROW(A10))</f>
+        <v>0.91279231299999997</v>
+      </c>
+      <c r="C11" s="5" cm="1">
+        <f t="array" ref="C11">INDEX($B$2:$M$13, COLUMN(B10), ROW(B10))</f>
+        <v>0.831354963</v>
+      </c>
+      <c r="D11" s="5" cm="1">
+        <f t="array" ref="D11">INDEX($B$2:$M$13, COLUMN(C10), ROW(C10))</f>
+        <v>1.8682599204038386</v>
+      </c>
+      <c r="E11" s="5" cm="1">
+        <f t="array" ref="E11">INDEX($B$2:$M$13, COLUMN(D10), ROW(D10))</f>
+        <v>1.0001761108457747</v>
+      </c>
+      <c r="F11" s="5" cm="1">
+        <f t="array" ref="F11">INDEX($B$2:$M$13, COLUMN(E10), ROW(E10))</f>
+        <v>0.77464335699999998</v>
+      </c>
+      <c r="G11" s="5" cm="1">
+        <f t="array" ref="G11">INDEX($B$2:$M$13, COLUMN(F10), ROW(F10))</f>
+        <v>0.50116565400000002</v>
+      </c>
+      <c r="H11" s="5" cm="1">
+        <f t="array" ref="H11">INDEX($B$2:$M$13, COLUMN(G10), ROW(G10))</f>
+        <v>0.94194245899999995</v>
+      </c>
+      <c r="I11" s="5" cm="1">
+        <f t="array" ref="I11">INDEX($B$2:$M$13, COLUMN(H10), ROW(H10))</f>
+        <v>0.94581527099999996</v>
+      </c>
+      <c r="J11" s="5" cm="1">
+        <f t="array" ref="J11">INDEX($B$2:$M$13, COLUMN(I10), ROW(I10))</f>
+        <v>0.89950992100000005</v>
+      </c>
+      <c r="K11" s="2"/>
+      <c r="L11">
+        <v>1.000176111</v>
+      </c>
+      <c r="M11">
+        <v>0.97954808599999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5" cm="1">
+        <f t="array" ref="B12">INDEX($B$2:$M$13, COLUMN(A11), ROW(A11))</f>
+        <v>0.60167079199999995</v>
+      </c>
+      <c r="C12" s="5" cm="1">
+        <f t="array" ref="C12">INDEX($B$2:$M$13, COLUMN(B11), ROW(B11))</f>
+        <v>0.944073524</v>
+      </c>
+      <c r="D12" s="5" cm="1">
+        <f t="array" ref="D12">INDEX($B$2:$M$13, COLUMN(C11), ROW(C11))</f>
+        <v>0.94194245855622349</v>
+      </c>
+      <c r="E12" s="5" cm="1">
+        <f t="array" ref="E12">INDEX($B$2:$M$13, COLUMN(D11), ROW(D11))</f>
+        <v>1.9999999901784853</v>
+      </c>
+      <c r="F12" s="5" cm="1">
+        <f t="array" ref="F12">INDEX($B$2:$M$13, COLUMN(E11), ROW(E11))</f>
+        <v>1.727029135</v>
+      </c>
+      <c r="G12" s="5" cm="1">
+        <f t="array" ref="G12">INDEX($B$2:$M$13, COLUMN(F11), ROW(F11))</f>
+        <v>0.42898139499999999</v>
+      </c>
+      <c r="H12" s="5" cm="1">
+        <f t="array" ref="H12">INDEX($B$2:$M$13, COLUMN(G11), ROW(G11))</f>
+        <v>0.99999999299999998</v>
+      </c>
+      <c r="I12" s="5" cm="1">
+        <f t="array" ref="I12">INDEX($B$2:$M$13, COLUMN(H11), ROW(H11))</f>
+        <v>0.59780924599999996</v>
+      </c>
+      <c r="J12" s="5" cm="1">
+        <f t="array" ref="J12">INDEX($B$2:$M$13, COLUMN(I11), ROW(I11))</f>
+        <v>1.000176111</v>
+      </c>
+      <c r="K12" s="5" cm="1">
+        <f t="array" ref="K12">INDEX($B$2:$M$13, COLUMN(J11), ROW(J11))</f>
+        <v>1.000176111</v>
+      </c>
+      <c r="L12" s="2"/>
+      <c r="M12">
+        <v>0.60721985000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" s="5" cm="1">
+        <f t="array" ref="B13">INDEX($B$2:$M$13, COLUMN(A12), ROW(A12))</f>
+        <v>0.34988060900000001</v>
+      </c>
+      <c r="C13" s="5" cm="1">
+        <f t="array" ref="C13">INDEX($B$2:$M$13, COLUMN(B12), ROW(B12))</f>
+        <v>1.300679519</v>
+      </c>
+      <c r="D13" s="5" cm="1">
+        <f t="array" ref="D13">INDEX($B$2:$M$13, COLUMN(C12), ROW(C12))</f>
+        <v>0.97954808599999998</v>
+      </c>
+      <c r="E13" s="5" cm="1">
+        <f t="array" ref="E13">INDEX($B$2:$M$13, COLUMN(D12), ROW(D12))</f>
+        <v>0.60721985043626692</v>
+      </c>
+      <c r="F13" s="5" cm="1">
+        <f t="array" ref="F13">INDEX($B$2:$M$13, COLUMN(E12), ROW(E12))</f>
+        <v>0.59641437900000005</v>
+      </c>
+      <c r="G13" s="5" cm="1">
+        <f t="array" ref="G13">INDEX($B$2:$M$13, COLUMN(F12), ROW(F12))</f>
+        <v>0.29768254</v>
+      </c>
+      <c r="H13" s="5" cm="1">
+        <f t="array" ref="H13">INDEX($B$2:$M$13, COLUMN(G12), ROW(G12))</f>
+        <v>1.4787779750000001</v>
+      </c>
+      <c r="I13" s="5" cm="1">
+        <f t="array" ref="I13">INDEX($B$2:$M$13, COLUMN(H12), ROW(H12))</f>
+        <v>0.388801124</v>
+      </c>
+      <c r="J13" s="5" cm="1">
+        <f t="array" ref="J13">INDEX($B$2:$M$13, COLUMN(I12), ROW(I12))</f>
+        <v>1.414274295</v>
+      </c>
+      <c r="K13" s="5" cm="1">
+        <f t="array" ref="K13">INDEX($B$2:$M$13, COLUMN(J12), ROW(J12))</f>
+        <v>0.97954808599999998</v>
+      </c>
+      <c r="L13" s="5" cm="1">
+        <f t="array" ref="L13">INDEX($B$2:$M$13, COLUMN(K12), ROW(K12))</f>
+        <v>0.60721985000000001</v>
+      </c>
+      <c r="M13" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
simple example new metrics
</commit_message>
<xml_diff>
--- a/ppm_output_handcalc.xlsx
+++ b/ppm_output_handcalc.xlsx
@@ -8,18 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drirpy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD08B68-E852-D74A-BDD5-1ED771684476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74053477-00C3-F940-8A7A-132A77FD835E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="1" xr2:uid="{BF39720B-7314-BE4F-87DC-079655431D8B}"/>
-    <workbookView xWindow="0" yWindow="9940" windowWidth="29400" windowHeight="9180" xr2:uid="{B4BFB160-4B0E-D64D-A7FA-99F45914B7D7}"/>
+    <workbookView xWindow="-4520" yWindow="-20940" windowWidth="18960" windowHeight="20800" activeTab="2" xr2:uid="{BF39720B-7314-BE4F-87DC-079655431D8B}"/>
+    <workbookView xWindow="13460" yWindow="-21100" windowWidth="20280" windowHeight="21100" activeTab="3" xr2:uid="{4F083981-888D-6D4A-9A91-0CE6B4D6ABC5}"/>
   </bookViews>
   <sheets>
     <sheet name="PPM" sheetId="1" r:id="rId1"/>
-    <sheet name="Information Content" sheetId="2" r:id="rId2"/>
-    <sheet name="KL" sheetId="9" r:id="rId3"/>
-    <sheet name="JSD" sheetId="10" r:id="rId4"/>
-    <sheet name="Pearson Correlation" sheetId="8" r:id="rId5"/>
+    <sheet name="KL" sheetId="9" r:id="rId2"/>
+    <sheet name="Information Content" sheetId="2" r:id="rId3"/>
+    <sheet name="Pearson Correlation" sheetId="8" r:id="rId4"/>
+    <sheet name="JSD" sheetId="10" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="PPM">PPM!$A$1:$M$5</definedName>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -248,7 +247,7 @@
       <name val="Calibri (Body)"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -303,8 +302,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -327,11 +332,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -354,8 +368,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -369,11 +381,12 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,8 +463,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>163904</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="7" name="Ink 6">
@@ -470,7 +483,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="7" name="Ink 6">
@@ -515,8 +528,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>129344</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="8" name="Ink 7">
@@ -535,7 +548,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="8" name="Ink 7">
@@ -580,8 +593,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>3239</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="9" name="Ink 8">
@@ -600,7 +613,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="9" name="Ink 8">
@@ -645,8 +658,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>25559</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="10" name="Ink 9">
@@ -665,7 +678,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="10" name="Ink 9">
@@ -710,8 +723,8 @@
       <xdr:row>26</xdr:row>
       <xdr:rowOff>59908</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="13" name="Ink 12">
@@ -730,7 +743,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="13" name="Ink 12">
@@ -775,8 +788,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>44999</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="14" name="Ink 13">
@@ -795,7 +808,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="14" name="Ink 13">
@@ -840,8 +853,8 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>72253</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="15" name="Ink 14">
@@ -860,7 +873,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="15" name="Ink 14">
@@ -905,8 +918,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>138344</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="16" name="Ink 15">
@@ -925,7 +938,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="16" name="Ink 15">
@@ -970,8 +983,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>134384</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="19" name="Ink 18">
@@ -990,7 +1003,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="19" name="Ink 18">
@@ -1035,8 +1048,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>111704</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="26" name="Ink 25">
@@ -1055,7 +1068,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="26" name="Ink 25">
@@ -1100,8 +1113,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>173519</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="27" name="Ink 26">
@@ -1120,7 +1133,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="27" name="Ink 26">
@@ -1165,8 +1178,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>65519</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="35" name="Ink 34">
@@ -1185,7 +1198,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="35" name="Ink 34">
@@ -1230,8 +1243,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>26279</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="36" name="Ink 35">
@@ -1250,7 +1263,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="36" name="Ink 35">
@@ -1295,8 +1308,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>4319</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId28">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="39" name="Ink 38">
@@ -1315,7 +1328,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="39" name="Ink 38">
@@ -1360,8 +1373,8 @@
       <xdr:row>26</xdr:row>
       <xdr:rowOff>9508</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId30">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="42" name="Ink 41">
@@ -1380,7 +1393,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="42" name="Ink 41">
@@ -1425,8 +1438,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>155549</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:aink="http://schemas.microsoft.com/office/drawing/2016/ink" Requires="xdr14 aink">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:aink="http://schemas.microsoft.com/office/drawing/2016/ink">
+      <mc:Choice Requires="xdr14 aink">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="43" name="Ink 42">
@@ -1445,7 +1458,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="43" name="Ink 42">
@@ -1490,8 +1503,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>58424</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId34">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="46" name="Ink 45">
@@ -1510,7 +1523,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="46" name="Ink 45">
@@ -2581,6 +2594,660 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06ED23D0-37BA-E443-BEB2-C0C6BD468A8C}">
+  <dimension ref="A1:T13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="2" max="9" width="5.5" customWidth="1"/>
+    <col min="10" max="10" width="7.1640625" customWidth="1"/>
+    <col min="11" max="11" width="8.1640625" customWidth="1"/>
+    <col min="12" max="12" width="7.5" customWidth="1"/>
+    <col min="13" max="13" width="6.1640625" customWidth="1"/>
+    <col min="15" max="15" width="4.1640625" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" customWidth="1"/>
+    <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="15">
+        <v>0</v>
+      </c>
+      <c r="C1" s="15">
+        <v>1</v>
+      </c>
+      <c r="D1" s="15">
+        <v>2</v>
+      </c>
+      <c r="E1" s="15">
+        <v>3</v>
+      </c>
+      <c r="F1" s="15">
+        <v>4</v>
+      </c>
+      <c r="G1" s="15">
+        <v>5</v>
+      </c>
+      <c r="H1" s="15">
+        <v>6</v>
+      </c>
+      <c r="I1" s="15">
+        <v>7</v>
+      </c>
+      <c r="J1" s="15">
+        <v>8</v>
+      </c>
+      <c r="K1" s="15">
+        <v>9</v>
+      </c>
+      <c r="L1" s="15">
+        <v>10</v>
+      </c>
+      <c r="M1" s="15">
+        <v>11</v>
+      </c>
+      <c r="P1" s="17">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="18">
+        <v>9</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" s="7"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A2" s="16">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="5">
+        <v>31.020705939999999</v>
+      </c>
+      <c r="D2" s="20">
+        <v>1.8600792660000001</v>
+      </c>
+      <c r="E2">
+        <v>4.9999999900000001</v>
+      </c>
+      <c r="F2">
+        <v>7.1966930930000004</v>
+      </c>
+      <c r="G2">
+        <v>4.6510474650000004</v>
+      </c>
+      <c r="H2">
+        <v>33.219280939999997</v>
+      </c>
+      <c r="I2" s="20">
+        <v>7.1603760000000004E-3</v>
+      </c>
+      <c r="J2">
+        <v>32.66223961</v>
+      </c>
+      <c r="K2" s="20">
+        <v>1.9307599209999999</v>
+      </c>
+      <c r="L2">
+        <v>4.9999999900000001</v>
+      </c>
+      <c r="M2" s="10">
+        <v>25.116701679999998</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" cm="1">
+        <f t="array" ref="P2">INDEX(PPM!$B$2:$M$5, ROW(A1), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>3.1250000100000001E-2</v>
+      </c>
+      <c r="Q2" cm="1">
+        <f t="array" ref="Q2">INDEX(PPM!$B$2:$M$5, ROW(B1), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1.5625000100000001E-2</v>
+      </c>
+      <c r="R2" s="5">
+        <f>P2*LOG(P2/Q2, 2)</f>
+        <v>3.1249999955730495E-2</v>
+      </c>
+      <c r="S2">
+        <f>Q2 * LOG(Q2/P2, 2)</f>
+        <v>-1.5625000027865248E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3" s="16">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5">
+        <v>24.515638259999999</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3">
+        <v>6.3091861807209408</v>
+      </c>
+      <c r="E3">
+        <v>4.4150374963453638</v>
+      </c>
+      <c r="F3">
+        <v>3.5609922491450261</v>
+      </c>
+      <c r="G3">
+        <v>19.486305897411111</v>
+      </c>
+      <c r="H3" s="20">
+        <v>9.3109404381863367E-2</v>
+      </c>
+      <c r="I3">
+        <v>25.043545593782468</v>
+      </c>
+      <c r="J3" s="20">
+        <v>4.4524455658293112E-2</v>
+      </c>
+      <c r="K3">
+        <v>5.8591198767729322</v>
+      </c>
+      <c r="L3">
+        <v>4.4150374963453638</v>
+      </c>
+      <c r="M3" s="20">
+        <v>0.69197659349035723</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" cm="1">
+        <f t="array" ref="P3">INDEX(PPM!$B$2:$M$5, ROW(A2), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.25000000010000001</v>
+      </c>
+      <c r="Q3" cm="1">
+        <f t="array" ref="Q3">INDEX(PPM!$B$2:$M$5, ROW(B2), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.98437500010000001</v>
+      </c>
+      <c r="R3" s="5">
+        <f t="shared" ref="R3:R5" si="0">P3*LOG(P3/Q3, 2)</f>
+        <v>-0.49431998096507751</v>
+      </c>
+      <c r="S3">
+        <f t="shared" ref="S3:S4" si="1">Q3 * LOG(Q3/P3, 2)</f>
+        <v>1.9463849244691667</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="16">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5">
+        <v>4.3575927019999998</v>
+      </c>
+      <c r="C4">
+        <v>32.312589736277587</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="F4">
+        <v>32.770416460439137</v>
+      </c>
+      <c r="G4">
+        <v>10.26726996944552</v>
+      </c>
+      <c r="H4">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="I4">
+        <v>4.0101324655174384</v>
+      </c>
+      <c r="J4">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="K4" s="20">
+        <v>0.42530126497041992</v>
+      </c>
+      <c r="L4">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="M4">
+        <v>24.65327670241172</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="P4" cm="1">
+        <f t="array" ref="P4">INDEX(PPM!$B$2:$M$5, ROW(A3), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>0.71875000010000001</v>
+      </c>
+      <c r="Q4" cm="1">
+        <f t="array" ref="Q4">INDEX(PPM!$B$2:$M$5, ROW(B3), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="R4" s="5">
+        <f t="shared" si="0"/>
+        <v>23.533918341337451</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="1"/>
+        <v>-3.2742842905131364E-9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="16">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5">
+        <v>31.182488580000001</v>
+      </c>
+      <c r="C5">
+        <v>31.274132205425509</v>
+      </c>
+      <c r="D5">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>2.6654431003916672</v>
+      </c>
+      <c r="G5">
+        <v>28.50137308568231</v>
+      </c>
+      <c r="H5">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="I5">
+        <v>31.779380872428789</v>
+      </c>
+      <c r="J5">
+        <v>32.584114609028987</v>
+      </c>
+      <c r="K5">
+        <v>32.584114609028987</v>
+      </c>
+      <c r="L5" s="20">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>32.433720656908612</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P5" cm="1">
+        <f t="array" ref="P5">INDEX(PPM!$B$2:$M$5, ROW(A4), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="Q5" cm="1">
+        <f t="array" ref="Q5">INDEX(PPM!$B$2:$M$5, ROW(B4), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
+        <v>1E-10</v>
+      </c>
+      <c r="R5" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <f>Q5 * LOG(Q5/P5, 2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A6" s="16">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5">
+        <v>31.186926669999998</v>
+      </c>
+      <c r="C6">
+        <v>3.339311110840403</v>
+      </c>
+      <c r="D6">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="E6" s="20">
+        <v>0.1420190048575036</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>23.857774328148071</v>
+      </c>
+      <c r="H6">
+        <v>3.415037497884239</v>
+      </c>
+      <c r="I6">
+        <v>31.781599919379691</v>
+      </c>
+      <c r="J6">
+        <v>3.247781508770196</v>
+      </c>
+      <c r="K6">
+        <v>32.586333655979892</v>
+      </c>
+      <c r="L6" s="20">
+        <v>0.1420190048575036</v>
+      </c>
+      <c r="M6">
+        <v>9.6148467646344109</v>
+      </c>
+      <c r="R6">
+        <f xml:space="preserve"> SUM(R2:R5)</f>
+        <v>23.070848360328103</v>
+      </c>
+      <c r="S6">
+        <f xml:space="preserve"> SUM(S2:S5)</f>
+        <v>1.930759921167017</v>
+      </c>
+      <c r="T6">
+        <f>AVERAGE(R6:S6)</f>
+        <v>12.50080414074756</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7" s="16">
+        <v>5</v>
+      </c>
+      <c r="B7" s="19">
+        <v>0.318100151</v>
+      </c>
+      <c r="C7">
+        <v>2.324622217424098</v>
+      </c>
+      <c r="D7">
+        <v>2.5318630882687709</v>
+      </c>
+      <c r="E7">
+        <v>3.415037497884239</v>
+      </c>
+      <c r="F7" s="20">
+        <v>2.8970824849101051</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>2.6780719043335819</v>
+      </c>
+      <c r="I7" s="20">
+        <v>0.35433235746951702</v>
+      </c>
+      <c r="J7">
+        <v>2.573471916572311</v>
+      </c>
+      <c r="K7">
+        <v>2.573471916572311</v>
+      </c>
+      <c r="L7">
+        <v>3.415037497884239</v>
+      </c>
+      <c r="M7" s="20">
+        <v>1.892511612224304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="16">
+        <v>6</v>
+      </c>
+      <c r="B8" s="5">
+        <v>32.220591110000001</v>
+      </c>
+      <c r="C8" s="20">
+        <v>1.688210110206448</v>
+      </c>
+      <c r="D8">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="E8">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="F8">
+        <v>29.65610887146871</v>
+      </c>
+      <c r="G8">
+        <v>26.425168026368691</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>32.298432137257187</v>
+      </c>
+      <c r="J8" s="20">
+        <v>0.4029361896679044</v>
+      </c>
+      <c r="K8">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="L8">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="M8">
+        <v>7.0002086803167911</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="16">
+        <v>7</v>
+      </c>
+      <c r="B9" s="19">
+        <v>8.9494190000000001E-3</v>
+      </c>
+      <c r="C9">
+        <v>31.067580940164301</v>
+      </c>
+      <c r="D9" s="20">
+        <v>1.859594473605175</v>
+      </c>
+      <c r="E9">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="F9">
+        <v>8.1029430921547796</v>
+      </c>
+      <c r="G9">
+        <v>4.7263752422845942</v>
+      </c>
+      <c r="H9">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>32.677864608886978</v>
+      </c>
+      <c r="K9" s="20">
+        <v>1.9463849242714379</v>
+      </c>
+      <c r="L9">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="M9">
+        <v>25.116701684381109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="16">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5">
+        <v>31.369988580000001</v>
+      </c>
+      <c r="C10" s="20">
+        <v>0.43360638701186949</v>
+      </c>
+      <c r="D10">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="E10">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="F10">
+        <v>4.9907655103560211</v>
+      </c>
+      <c r="G10">
+        <v>23.876910448498951</v>
+      </c>
+      <c r="H10" s="20">
+        <v>2.2720076497793468E-2</v>
+      </c>
+      <c r="I10">
+        <v>31.873130872286779</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>32.677864608886978</v>
+      </c>
+      <c r="L10">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="M10">
+        <v>7.0176037388854144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="16">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5">
+        <v>23.070848359999999</v>
+      </c>
+      <c r="C11">
+        <v>31.03668594136634</v>
+      </c>
+      <c r="D11" s="20">
+        <v>0.42530126497041992</v>
+      </c>
+      <c r="E11">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="F11">
+        <v>8.1029430921547796</v>
+      </c>
+      <c r="G11">
+        <v>23.876910448498951</v>
+      </c>
+      <c r="H11">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="I11">
+        <v>23.573990654156749</v>
+      </c>
+      <c r="J11">
+        <v>32.677864608886978</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>5.9999999909110224</v>
+      </c>
+      <c r="M11">
+        <v>24.65327670241172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12" s="16">
+        <v>10</v>
+      </c>
+      <c r="B12" s="5">
+        <v>31.182488580000001</v>
+      </c>
+      <c r="C12">
+        <v>31.274132205425509</v>
+      </c>
+      <c r="D12">
+        <v>33.1031658738574</v>
+      </c>
+      <c r="E12" s="20">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>2.6654431003916672</v>
+      </c>
+      <c r="G12">
+        <v>28.50137308568231</v>
+      </c>
+      <c r="H12">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="I12">
+        <v>31.779380872428789</v>
+      </c>
+      <c r="J12">
+        <v>32.584114609028987</v>
+      </c>
+      <c r="K12">
+        <v>32.584114609028987</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>32.433720656908612</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A13" s="16">
+        <v>11</v>
+      </c>
+      <c r="B13" s="5">
+        <v>24.43904822</v>
+      </c>
+      <c r="C13" s="20">
+        <v>1.5630732009148851</v>
+      </c>
+      <c r="D13">
+        <v>2.4633407591518521</v>
+      </c>
+      <c r="E13">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="F13">
+        <v>29.692229823578771</v>
+      </c>
+      <c r="G13">
+        <v>21.621905309297279</v>
+      </c>
+      <c r="H13">
+        <v>0.38529015584062748</v>
+      </c>
+      <c r="I13">
+        <v>24.516889250982771</v>
+      </c>
+      <c r="J13">
+        <v>0.78220618682352216</v>
+      </c>
+      <c r="K13">
+        <v>2.4633407591518521</v>
+      </c>
+      <c r="L13">
+        <v>33.219280949017893</v>
+      </c>
+      <c r="M13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67C6B552-D222-D944-AA0C-60A0FCCF6FC4}">
   <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2649,10 +3316,10 @@
       <c r="R1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="S1" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="25" t="s">
+      <c r="T1" s="22" t="s">
         <v>27</v>
       </c>
       <c r="U1" s="6" t="s">
@@ -2686,13 +3353,13 @@
       <c r="H2">
         <v>0.500655077</v>
       </c>
-      <c r="I2" s="14">
+      <c r="I2" s="12">
         <v>1.0382551289999999</v>
       </c>
       <c r="J2">
         <v>0.46412009799999998</v>
       </c>
-      <c r="K2" s="15">
+      <c r="K2" s="13">
         <v>0.91279231299999997</v>
       </c>
       <c r="L2">
@@ -2750,13 +3417,13 @@
       <c r="G3" s="5">
         <v>0.43011038600000001</v>
       </c>
-      <c r="H3" s="15">
+      <c r="H3" s="13">
         <v>1.7740252299999999</v>
       </c>
       <c r="I3">
         <v>0.41379671899999998</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="12">
         <v>1.7338225279999999</v>
       </c>
       <c r="K3">
@@ -2765,7 +3432,7 @@
       <c r="L3">
         <v>0.944073524</v>
       </c>
-      <c r="M3" s="15">
+      <c r="M3" s="13">
         <v>1.300679519</v>
       </c>
       <c r="O3" s="3" t="s">
@@ -2821,13 +3488,13 @@
       <c r="H4">
         <v>0.94194245855622349</v>
       </c>
-      <c r="I4" s="12">
+      <c r="I4">
         <v>0.984975614485744</v>
       </c>
       <c r="J4">
         <v>0.88388492366776417</v>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="12">
         <v>1.8682599204038386</v>
       </c>
       <c r="L4">
@@ -2881,7 +3548,7 @@
         <v>0.94194245855622349</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="15">
+      <c r="F5" s="13">
         <v>1.7270291352821832</v>
       </c>
       <c r="G5">
@@ -2899,7 +3566,7 @@
       <c r="K5">
         <v>1.0001761108457747</v>
       </c>
-      <c r="L5" s="14">
+      <c r="L5" s="12">
         <v>1.9999999901784853</v>
       </c>
       <c r="M5">
@@ -2969,7 +3636,7 @@
       <c r="K6">
         <v>0.77464335699999998</v>
       </c>
-      <c r="L6" s="15">
+      <c r="L6" s="13">
         <v>1.727029135</v>
       </c>
       <c r="M6">
@@ -3048,23 +3715,23 @@
         <f t="array" ref="B8">INDEX($B$2:$M$13, COLUMN(A7), ROW(A7))</f>
         <v>0.500655077</v>
       </c>
-      <c r="C8" s="13" cm="1">
+      <c r="C8" s="5" cm="1">
         <f t="array" ref="C8">INDEX($B$2:$M$13, COLUMN(B7), ROW(B7))</f>
         <v>1.7740252299999999</v>
       </c>
-      <c r="D8" s="13" cm="1">
+      <c r="D8" s="5" cm="1">
         <f t="array" ref="D8">INDEX($B$2:$M$13, COLUMN(C7), ROW(C7))</f>
         <v>0.94194245855622349</v>
       </c>
-      <c r="E8" s="13" cm="1">
+      <c r="E8" s="5" cm="1">
         <f t="array" ref="E8">INDEX($B$2:$M$13, COLUMN(D7), ROW(D7))</f>
         <v>0.99999999344468282</v>
       </c>
-      <c r="F8" s="13" cm="1">
+      <c r="F8" s="5" cm="1">
         <f t="array" ref="F8">INDEX($B$2:$M$13, COLUMN(E7), ROW(E7))</f>
         <v>1.006349282</v>
       </c>
-      <c r="G8" s="13" cm="1">
+      <c r="G8" s="5" cm="1">
         <f t="array" ref="G8">INDEX($B$2:$M$13, COLUMN(F7), ROW(F7))</f>
         <v>0.52851445699999999</v>
       </c>
@@ -3072,7 +3739,7 @@
       <c r="I8">
         <v>0.53957559300000002</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="13">
         <v>1.9340855809999999</v>
       </c>
       <c r="K8">
@@ -3081,7 +3748,7 @@
       <c r="L8">
         <v>0.99999999299999998</v>
       </c>
-      <c r="M8" s="15">
+      <c r="M8" s="13">
         <v>1.4787779750000001</v>
       </c>
     </row>
@@ -3093,23 +3760,23 @@
         <f t="array" ref="B9">INDEX($B$2:$M$13, COLUMN(A8), ROW(A8))</f>
         <v>1.0382551289999999</v>
       </c>
-      <c r="C9" s="13" cm="1">
+      <c r="C9" s="5" cm="1">
         <f t="array" ref="C9">INDEX($B$2:$M$13, COLUMN(B8), ROW(B8))</f>
         <v>0.41379671899999998</v>
       </c>
-      <c r="D9" s="13" cm="1">
+      <c r="D9" s="5" cm="1">
         <f t="array" ref="D9">INDEX($B$2:$M$13, COLUMN(C8), ROW(C8))</f>
         <v>0.984975614485744</v>
       </c>
-      <c r="E9" s="13" cm="1">
+      <c r="E9" s="5" cm="1">
         <f t="array" ref="E9">INDEX($B$2:$M$13, COLUMN(D8), ROW(D8))</f>
         <v>0.59780924559747062</v>
       </c>
-      <c r="F9" s="13" cm="1">
+      <c r="F9" s="5" cm="1">
         <f t="array" ref="F9">INDEX($B$2:$M$13, COLUMN(E8), ROW(E8))</f>
         <v>0.37227649099999999</v>
       </c>
-      <c r="G9" s="13" cm="1">
+      <c r="G9" s="5" cm="1">
         <f t="array" ref="G9">INDEX($B$2:$M$13, COLUMN(F8), ROW(F8))</f>
         <v>0.62406583999999998</v>
       </c>
@@ -3121,7 +3788,7 @@
       <c r="J9">
         <v>0.49714305600000003</v>
       </c>
-      <c r="K9" s="15">
+      <c r="K9" s="13">
         <v>0.94581527099999996</v>
       </c>
       <c r="L9">
@@ -3139,23 +3806,23 @@
         <f t="array" ref="B10">INDEX($B$2:$M$13, COLUMN(A9), ROW(A9))</f>
         <v>0.46412009799999998</v>
       </c>
-      <c r="C10" s="13" cm="1">
+      <c r="C10" s="5" cm="1">
         <f t="array" ref="C10">INDEX($B$2:$M$13, COLUMN(B9), ROW(B9))</f>
         <v>1.7338225279999999</v>
       </c>
-      <c r="D10" s="13" cm="1">
+      <c r="D10" s="5" cm="1">
         <f t="array" ref="D10">INDEX($B$2:$M$13, COLUMN(C9), ROW(C9))</f>
         <v>0.88388492366776417</v>
       </c>
-      <c r="E10" s="13" cm="1">
+      <c r="E10" s="5" cm="1">
         <f t="array" ref="E10">INDEX($B$2:$M$13, COLUMN(D9), ROW(D9))</f>
         <v>1.000176111</v>
       </c>
-      <c r="F10" s="13" cm="1">
+      <c r="F10" s="5" cm="1">
         <f t="array" ref="F10">INDEX($B$2:$M$13, COLUMN(E9), ROW(E9))</f>
         <v>1.0044072390000001</v>
       </c>
-      <c r="G10" s="13" cm="1">
+      <c r="G10" s="5" cm="1">
         <f t="array" ref="G10">INDEX($B$2:$M$13, COLUMN(F9), ROW(F9))</f>
         <v>0.50116565400000002</v>
       </c>
@@ -3174,7 +3841,7 @@
       <c r="L10">
         <v>1.000176111</v>
       </c>
-      <c r="M10" s="15">
+      <c r="M10" s="13">
         <v>1.414274295</v>
       </c>
     </row>
@@ -3186,23 +3853,23 @@
         <f t="array" ref="B11">INDEX($B$2:$M$13, COLUMN(A10), ROW(A10))</f>
         <v>0.91279231299999997</v>
       </c>
-      <c r="C11" s="13" cm="1">
+      <c r="C11" s="5" cm="1">
         <f t="array" ref="C11">INDEX($B$2:$M$13, COLUMN(B10), ROW(B10))</f>
         <v>0.831354963</v>
       </c>
-      <c r="D11" s="13" cm="1">
+      <c r="D11" s="5" cm="1">
         <f t="array" ref="D11">INDEX($B$2:$M$13, COLUMN(C10), ROW(C10))</f>
         <v>1.8682599204038386</v>
       </c>
-      <c r="E11" s="13" cm="1">
+      <c r="E11" s="5" cm="1">
         <f t="array" ref="E11">INDEX($B$2:$M$13, COLUMN(D10), ROW(D10))</f>
         <v>1.0001761108457747</v>
       </c>
-      <c r="F11" s="13" cm="1">
+      <c r="F11" s="5" cm="1">
         <f t="array" ref="F11">INDEX($B$2:$M$13, COLUMN(E10), ROW(E10))</f>
         <v>0.77464335699999998</v>
       </c>
-      <c r="G11" s="13" cm="1">
+      <c r="G11" s="5" cm="1">
         <f t="array" ref="G11">INDEX($B$2:$M$13, COLUMN(F10), ROW(F10))</f>
         <v>0.50116565400000002</v>
       </c>
@@ -3234,23 +3901,23 @@
         <f t="array" ref="B12">INDEX($B$2:$M$13, COLUMN(A11), ROW(A11))</f>
         <v>0.60167079199999995</v>
       </c>
-      <c r="C12" s="13" cm="1">
+      <c r="C12" s="5" cm="1">
         <f t="array" ref="C12">INDEX($B$2:$M$13, COLUMN(B11), ROW(B11))</f>
         <v>0.944073524</v>
       </c>
-      <c r="D12" s="13" cm="1">
+      <c r="D12" s="5" cm="1">
         <f t="array" ref="D12">INDEX($B$2:$M$13, COLUMN(C11), ROW(C11))</f>
         <v>0.94194245855622349</v>
       </c>
-      <c r="E12" s="13" cm="1">
+      <c r="E12" s="5" cm="1">
         <f t="array" ref="E12">INDEX($B$2:$M$13, COLUMN(D11), ROW(D11))</f>
         <v>1.9999999901784853</v>
       </c>
-      <c r="F12" s="13" cm="1">
+      <c r="F12" s="5" cm="1">
         <f t="array" ref="F12">INDEX($B$2:$M$13, COLUMN(E11), ROW(E11))</f>
         <v>1.727029135</v>
       </c>
-      <c r="G12" s="13" cm="1">
+      <c r="G12" s="5" cm="1">
         <f t="array" ref="G12">INDEX($B$2:$M$13, COLUMN(F11), ROW(F11))</f>
         <v>0.42898139499999999</v>
       </c>
@@ -3283,23 +3950,23 @@
         <f t="array" ref="B13">INDEX($B$2:$M$13, COLUMN(A12), ROW(A12))</f>
         <v>0.34988060900000001</v>
       </c>
-      <c r="C13" s="13" cm="1">
+      <c r="C13" s="5" cm="1">
         <f t="array" ref="C13">INDEX($B$2:$M$13, COLUMN(B12), ROW(B12))</f>
         <v>1.300679519</v>
       </c>
-      <c r="D13" s="13" cm="1">
+      <c r="D13" s="5" cm="1">
         <f t="array" ref="D13">INDEX($B$2:$M$13, COLUMN(C12), ROW(C12))</f>
         <v>0.97954808599999998</v>
       </c>
-      <c r="E13" s="13" cm="1">
+      <c r="E13" s="5" cm="1">
         <f t="array" ref="E13">INDEX($B$2:$M$13, COLUMN(D12), ROW(D12))</f>
         <v>0.60721985043626692</v>
       </c>
-      <c r="F13" s="13" cm="1">
+      <c r="F13" s="5" cm="1">
         <f t="array" ref="F13">INDEX($B$2:$M$13, COLUMN(E12), ROW(E12))</f>
         <v>0.59641437900000005</v>
       </c>
-      <c r="G13" s="13" cm="1">
+      <c r="G13" s="5" cm="1">
         <f t="array" ref="G13">INDEX($B$2:$M$13, COLUMN(F12), ROW(F12))</f>
         <v>0.29768254</v>
       </c>
@@ -3326,7 +3993,7 @@
       <c r="M13" s="2"/>
     </row>
     <row r="16" spans="1:22" ht="32" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B16" t="s">
@@ -3338,8 +4005,9 @@
       <c r="D16" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="L16" s="23"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -3352,8 +4020,9 @@
       <c r="D17" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="L17" s="23"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -3367,7 +4036,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -3381,7 +4050,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -3395,7 +4064,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -3406,7 +4075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -3417,7 +4086,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -3428,7 +4097,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -3445,14 +4114,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06ED23D0-37BA-E443-BEB2-C0C6BD468A8C}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3125F5A-7234-5647-851D-0D6A6A07A661}">
   <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.5" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
     <col min="2" max="9" width="5.5" customWidth="1"/>
-    <col min="10" max="10" width="7.1640625" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" customWidth="1"/>
     <col min="11" max="11" width="8.1640625" customWidth="1"/>
     <col min="12" max="12" width="7.5" customWidth="1"/>
     <col min="13" max="13" width="6.1640625" customWidth="1"/>
@@ -3466,273 +4135,252 @@
   <sheetData>
     <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="17">
-        <v>0</v>
-      </c>
-      <c r="C1" s="17">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1">
         <v>1</v>
       </c>
-      <c r="D1" s="17">
+      <c r="D1" s="1">
         <v>2</v>
       </c>
-      <c r="E1" s="17">
+      <c r="E1" s="1">
         <v>3</v>
       </c>
-      <c r="F1" s="17">
+      <c r="F1" s="1">
         <v>4</v>
       </c>
-      <c r="G1" s="17">
+      <c r="G1" s="1">
         <v>5</v>
       </c>
-      <c r="H1" s="17">
+      <c r="H1" s="1">
         <v>6</v>
       </c>
-      <c r="I1" s="17">
+      <c r="I1" s="1">
         <v>7</v>
       </c>
-      <c r="J1" s="17">
+      <c r="J1" s="1">
         <v>8</v>
       </c>
-      <c r="K1" s="17">
+      <c r="K1" s="1">
         <v>9</v>
       </c>
-      <c r="L1" s="17">
+      <c r="L1" s="1">
         <v>10</v>
       </c>
-      <c r="M1" s="17">
+      <c r="M1" s="1">
         <v>11</v>
       </c>
-      <c r="P1" s="19">
-        <v>0</v>
-      </c>
-      <c r="Q1" s="20">
+      <c r="P1" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q1" s="9">
         <v>9</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>17</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="S1" s="6"/>
       <c r="T1" s="7"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2" s="18">
+      <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="5">
-        <v>31.020705939999999</v>
-      </c>
-      <c r="D2" s="22">
-        <v>1.8600792660000001</v>
+        <v>-0.53587699799999999</v>
+      </c>
+      <c r="D2">
+        <v>1.5031991999999999E-2</v>
       </c>
       <c r="E2">
-        <v>4.9999999900000001</v>
+        <v>-0.43965200500000001</v>
       </c>
       <c r="F2">
-        <v>7.1966930930000004</v>
-      </c>
-      <c r="G2">
-        <v>4.6510474650000004</v>
+        <v>-0.50661061399999996</v>
+      </c>
+      <c r="G2" s="12">
+        <v>0.95141007099999997</v>
       </c>
       <c r="H2">
-        <v>33.219280939999997</v>
-      </c>
-      <c r="I2" s="22">
-        <v>7.1603760000000004E-3</v>
+        <v>-0.50245943400000004</v>
+      </c>
+      <c r="I2" s="21">
+        <v>0.99980301599999999</v>
       </c>
       <c r="J2">
-        <v>32.66223961</v>
-      </c>
-      <c r="K2" s="22">
-        <v>1.9307599209999999</v>
+        <v>-0.51208986300000003</v>
+      </c>
+      <c r="K2" s="24">
+        <v>-7.01493E-3</v>
       </c>
       <c r="L2">
-        <v>4.9999999900000001</v>
+        <v>-0.43965200500000001</v>
       </c>
       <c r="M2" s="10">
-        <v>25.116701679999998</v>
+        <v>-0.53271688299999997</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>0</v>
       </c>
       <c r="P2" cm="1">
         <f t="array" ref="P2">INDEX(PPM!$B$2:$M$5, ROW(A1), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>3.1250000100000001E-2</v>
+        <v>1.0000000001</v>
       </c>
       <c r="Q2" cm="1">
         <f t="array" ref="Q2">INDEX(PPM!$B$2:$M$5, ROW(B1), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
         <v>1.5625000100000001E-2</v>
       </c>
-      <c r="R2" s="5">
-        <f>P2*LOG(P2/Q2, 2)</f>
-        <v>3.1249999955730495E-2</v>
-      </c>
-      <c r="S2">
-        <f>Q2 * LOG(Q2/P2, 2)</f>
-        <v>-1.5625000027865248E-2</v>
-      </c>
+      <c r="R2" s="5"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3" s="18">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="5">
-        <v>24.515638259999999</v>
+      <c r="B3" s="5" cm="1">
+        <f t="array" ref="B3">INDEX($B$2:$M$13, COLUMN(A2), ROW(A2))</f>
+        <v>-0.53587699799999999</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3">
-        <v>6.3091861807209408</v>
+        <v>-0.3481711293029694</v>
       </c>
       <c r="E3">
-        <v>4.4150374963453638</v>
+        <v>-0.29518783809240762</v>
       </c>
       <c r="F3">
-        <v>3.5609922491450261</v>
+        <v>-0.19767811977548069</v>
       </c>
       <c r="G3">
-        <v>19.486305897411111</v>
-      </c>
-      <c r="H3" s="22">
-        <v>9.3109404381863367E-2</v>
+        <v>-0.30403879734200751</v>
+      </c>
+      <c r="H3" s="12">
+        <v>0.99909729815891835</v>
       </c>
       <c r="I3">
-        <v>25.043545593782468</v>
-      </c>
-      <c r="J3" s="22">
-        <v>4.4524455658293112E-2</v>
+        <v>-0.52043820617740066</v>
+      </c>
+      <c r="J3" s="12">
+        <v>0.99958808090207341</v>
       </c>
       <c r="K3">
-        <v>5.8591198767729322</v>
+        <v>-0.34708422671409428</v>
       </c>
       <c r="L3">
-        <v>4.4150374963453638</v>
-      </c>
-      <c r="M3" s="22">
-        <v>0.69197659349035723</v>
+        <v>-0.29518783809240762</v>
+      </c>
+      <c r="M3" s="12">
+        <v>0.94871716359144431</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="P3" cm="1">
         <f t="array" ref="P3">INDEX(PPM!$B$2:$M$5, ROW(A2), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>0.25000000010000001</v>
+        <v>1E-10</v>
       </c>
       <c r="Q3" cm="1">
         <f t="array" ref="Q3">INDEX(PPM!$B$2:$M$5, ROW(B2), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
         <v>0.98437500010000001</v>
       </c>
-      <c r="R3" s="5">
-        <f t="shared" ref="R3:R5" si="0">P3*LOG(P3/Q3, 2)</f>
-        <v>-0.49431998096507751</v>
-      </c>
-      <c r="S3">
-        <f t="shared" ref="S3:S5" si="1">Q3 * LOG(Q3/P3, 2)</f>
-        <v>1.9463849244691667</v>
-      </c>
+      <c r="R3" s="5"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="18">
+      <c r="A4">
         <v>2</v>
       </c>
-      <c r="B4" s="5">
-        <v>4.3575927019999998</v>
-      </c>
-      <c r="C4">
-        <v>32.312589736277587</v>
-      </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
+      <c r="B4" s="5" cm="1">
+        <f t="array" ref="B4">INDEX($B$2:$M$13, COLUMN(A3), ROW(A3))</f>
+        <v>1.5031991999999999E-2</v>
+      </c>
+      <c r="C4" s="5" cm="1">
+        <f t="array" ref="C4">INDEX($B$2:$M$13, COLUMN(B3), ROW(B3))</f>
+        <v>-0.3481711293029694</v>
+      </c>
+      <c r="D4" s="2"/>
       <c r="E4">
-        <v>33.219280949017893</v>
+        <v>-0.34038701134538812</v>
       </c>
       <c r="F4">
-        <v>32.770416460439137</v>
+        <v>-0.38704402483723771</v>
       </c>
       <c r="G4">
-        <v>10.26726996944552</v>
+        <v>-0.25608356496295148</v>
       </c>
       <c r="H4">
-        <v>33.219280949017893</v>
+        <v>-0.34038701134538812</v>
       </c>
       <c r="I4">
-        <v>4.0101324655174384</v>
+        <v>1.5040514489777961E-2</v>
       </c>
       <c r="J4">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="K4" s="22">
-        <v>0.42530126497041992</v>
+        <v>-0.34758995247793623</v>
+      </c>
+      <c r="K4" s="12">
+        <v>0.99966055668703313</v>
       </c>
       <c r="L4">
-        <v>33.219280949017893</v>
+        <v>-0.34038701134538812</v>
       </c>
       <c r="M4">
-        <v>24.65327670241172</v>
+        <v>-3.6364654371126022E-2</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="P4" cm="1">
         <f t="array" ref="P4">INDEX(PPM!$B$2:$M$5, ROW(A3), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>0.71875000010000001</v>
+        <v>1E-10</v>
       </c>
       <c r="Q4" cm="1">
         <f t="array" ref="Q4">INDEX(PPM!$B$2:$M$5, ROW(B3), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
         <v>1E-10</v>
       </c>
-      <c r="R4" s="5">
-        <f t="shared" si="0"/>
-        <v>23.533918341337451</v>
-      </c>
-      <c r="S4">
-        <f t="shared" si="1"/>
-        <v>-3.2742842905131364E-9</v>
-      </c>
+      <c r="R4" s="5"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="18">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="B5" s="5">
-        <v>31.182488580000001</v>
-      </c>
-      <c r="C5">
-        <v>31.274132205425509</v>
-      </c>
-      <c r="D5">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>2.6654431003916672</v>
+      <c r="B5" s="5" cm="1">
+        <f t="array" ref="B5">INDEX($B$2:$M$13, COLUMN(A4), ROW(A4))</f>
+        <v>-0.43965200500000001</v>
+      </c>
+      <c r="C5" s="5" cm="1">
+        <f t="array" ref="C5">INDEX($B$2:$M$13, COLUMN(B4), ROW(B4))</f>
+        <v>-0.29518783809240762</v>
+      </c>
+      <c r="D5" s="5" cm="1">
+        <f t="array" ref="D5">INDEX($B$2:$M$13, COLUMN(C4), ROW(C4))</f>
+        <v>-0.34038701134538812</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="12">
+        <v>0.99493667632618188</v>
       </c>
       <c r="G5">
-        <v>28.50137308568231</v>
+        <v>-0.45083481733371611</v>
       </c>
       <c r="H5">
-        <v>33.219280949017893</v>
+        <v>-0.33333333333333331</v>
       </c>
       <c r="I5">
-        <v>31.779380872428789</v>
+        <v>-0.45611882530944092</v>
       </c>
       <c r="J5">
-        <v>32.584114609028987</v>
+        <v>-0.31911282313630129</v>
       </c>
       <c r="K5">
-        <v>32.584114609028987</v>
-      </c>
-      <c r="L5" s="22">
-        <v>0</v>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0.99999999999999944</v>
       </c>
       <c r="M5">
-        <v>32.433720656908612</v>
+        <v>-0.46159181056844312</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>3</v>
@@ -3745,361 +4393,391 @@
         <f t="array" ref="Q5">INDEX(PPM!$B$2:$M$5, ROW(B4), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
         <v>1E-10</v>
       </c>
-      <c r="R5" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <f>Q5 * LOG(Q5/P5, 2)</f>
-        <v>0</v>
-      </c>
+      <c r="R5" s="5"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6" s="18">
+      <c r="A6">
         <v>4</v>
       </c>
-      <c r="B6" s="5">
-        <v>31.186926669999998</v>
-      </c>
-      <c r="C6">
-        <v>3.339311110840403</v>
-      </c>
-      <c r="D6">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="E6" s="22">
-        <v>0.1420190048575036</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
+      <c r="B6" s="5" cm="1">
+        <f t="array" ref="B6">INDEX($B$2:$M$13, COLUMN(A5), ROW(A5))</f>
+        <v>-0.50661061399999996</v>
+      </c>
+      <c r="C6" s="5" cm="1">
+        <f t="array" ref="C6">INDEX($B$2:$M$13, COLUMN(B5), ROW(B5))</f>
+        <v>-0.19767811977548069</v>
+      </c>
+      <c r="D6" s="5" cm="1">
+        <f t="array" ref="D6">INDEX($B$2:$M$13, COLUMN(C5), ROW(C5))</f>
+        <v>-0.38704402483723771</v>
+      </c>
+      <c r="E6" s="5" cm="1">
+        <f t="array" ref="E6">INDEX($B$2:$M$13, COLUMN(D5), ROW(D5))</f>
+        <v>0.99493667632618188</v>
+      </c>
+      <c r="F6" s="2"/>
       <c r="G6">
-        <v>23.857774328148071</v>
+        <v>-0.49340730420314183</v>
       </c>
       <c r="H6">
-        <v>3.415037497884239</v>
+        <v>-0.23688968483956721</v>
       </c>
       <c r="I6">
-        <v>31.781599919379691</v>
+        <v>-0.52188075027265435</v>
       </c>
       <c r="J6">
-        <v>3.247781508770196</v>
+        <v>-0.22224793613700761</v>
       </c>
       <c r="K6">
-        <v>32.586333655979892</v>
-      </c>
-      <c r="L6" s="22">
-        <v>0.1420190048575036</v>
+        <v>-0.36512160936794091</v>
+      </c>
+      <c r="L6" s="12">
+        <v>0.99493667632618188</v>
       </c>
       <c r="M6">
-        <v>9.6148467646344109</v>
+        <v>-0.37416950215763012</v>
       </c>
       <c r="R6">
-        <f xml:space="preserve"> SUM(R2:R5)</f>
-        <v>23.070848360328103</v>
-      </c>
-      <c r="S6">
-        <f xml:space="preserve"> SUM(S2:S5)</f>
-        <v>1.930759921167017</v>
-      </c>
-      <c r="T6">
-        <f>AVERAGE(R6:S6)</f>
-        <v>12.50080414074756</v>
-      </c>
+        <f>CORREL(P2:P5, Q2:Q5)</f>
+        <v>-0.3191128231363014</v>
+      </c>
+      <c r="S6" s="3"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="18">
+      <c r="A7">
         <v>5</v>
       </c>
-      <c r="B7" s="21">
-        <v>0.318100151</v>
-      </c>
-      <c r="C7">
-        <v>2.324622217424098</v>
-      </c>
-      <c r="D7">
-        <v>2.5318630882687709</v>
-      </c>
-      <c r="E7">
-        <v>3.415037497884239</v>
-      </c>
-      <c r="F7" s="22">
-        <v>2.8970824849101051</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0</v>
-      </c>
+      <c r="B7" s="5" cm="1">
+        <f t="array" ref="B7">INDEX($B$2:$M$13, COLUMN(A6), ROW(A6))</f>
+        <v>0.95141007099999997</v>
+      </c>
+      <c r="C7" s="5" cm="1">
+        <f t="array" ref="C7">INDEX($B$2:$M$13, COLUMN(B6), ROW(B6))</f>
+        <v>-0.30403879734200751</v>
+      </c>
+      <c r="D7" s="5" cm="1">
+        <f t="array" ref="D7">INDEX($B$2:$M$13, COLUMN(C6), ROW(C6))</f>
+        <v>-0.25608356496295148</v>
+      </c>
+      <c r="E7" s="5" cm="1">
+        <f t="array" ref="E7">INDEX($B$2:$M$13, COLUMN(D6), ROW(D6))</f>
+        <v>-0.45083481733371611</v>
+      </c>
+      <c r="F7" s="5" cm="1">
+        <f t="array" ref="F7">INDEX($B$2:$M$13, COLUMN(E6), ROW(E6))</f>
+        <v>-0.49340730420314183</v>
+      </c>
+      <c r="G7" s="2"/>
       <c r="H7">
-        <v>2.6780719043335819</v>
-      </c>
-      <c r="I7" s="22">
-        <v>0.35433235746951702</v>
+        <v>-0.27050089040022968</v>
+      </c>
+      <c r="I7" s="12">
+        <v>0.95414290742954877</v>
       </c>
       <c r="J7">
-        <v>2.573471916572311</v>
+        <v>-0.27910231237535182</v>
       </c>
       <c r="K7">
-        <v>2.573471916572311</v>
+        <v>-0.27910231237535171</v>
       </c>
       <c r="L7">
-        <v>3.415037497884239</v>
-      </c>
-      <c r="M7" s="22">
-        <v>1.892511612224304</v>
+        <v>-0.45083481733371611</v>
+      </c>
+      <c r="M7">
+        <v>-0.37458298728065398</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="18">
+      <c r="A8">
         <v>6</v>
       </c>
-      <c r="B8" s="5">
-        <v>32.220591110000001</v>
-      </c>
-      <c r="C8" s="22">
-        <v>1.688210110206448</v>
-      </c>
-      <c r="D8">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="E8">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="F8">
-        <v>29.65610887146871</v>
-      </c>
-      <c r="G8">
-        <v>26.425168026368691</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0</v>
-      </c>
+      <c r="B8" s="5" cm="1">
+        <f t="array" ref="B8">INDEX($B$2:$M$13, COLUMN(A7), ROW(A7))</f>
+        <v>-0.50245943400000004</v>
+      </c>
+      <c r="C8" s="5" cm="1">
+        <f t="array" ref="C8">INDEX($B$2:$M$13, COLUMN(B7), ROW(B7))</f>
+        <v>0.99909729815891835</v>
+      </c>
+      <c r="D8" s="5" cm="1">
+        <f t="array" ref="D8">INDEX($B$2:$M$13, COLUMN(C7), ROW(C7))</f>
+        <v>-0.34038701134538812</v>
+      </c>
+      <c r="E8" s="5" cm="1">
+        <f t="array" ref="E8">INDEX($B$2:$M$13, COLUMN(D7), ROW(D7))</f>
+        <v>-0.33333333333333331</v>
+      </c>
+      <c r="F8" s="5" cm="1">
+        <f t="array" ref="F8">INDEX($B$2:$M$13, COLUMN(E7), ROW(E7))</f>
+        <v>-0.23688968483956721</v>
+      </c>
+      <c r="G8" s="5" cm="1">
+        <f t="array" ref="G8">INDEX($B$2:$M$13, COLUMN(F7), ROW(F7))</f>
+        <v>-0.27050089040022968</v>
+      </c>
+      <c r="H8" s="2"/>
       <c r="I8">
-        <v>32.298432137257187</v>
-      </c>
-      <c r="J8" s="22">
-        <v>0.4029361896679044</v>
+        <v>-0.48652674699673709</v>
+      </c>
+      <c r="J8" s="12">
+        <v>0.99988684582707787</v>
       </c>
       <c r="K8">
-        <v>33.1031658738574</v>
+        <v>-0.34038701134538812</v>
       </c>
       <c r="L8">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="M8">
-        <v>7.0002086803167911</v>
+        <v>-0.33333333333333331</v>
+      </c>
+      <c r="M8" s="12">
+        <v>0.95203310929741403</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="18">
+      <c r="A9">
         <v>7</v>
       </c>
-      <c r="B9" s="21">
-        <v>8.9494190000000001E-3</v>
-      </c>
-      <c r="C9">
-        <v>31.067580940164301</v>
-      </c>
-      <c r="D9" s="22">
-        <v>1.859594473605175</v>
-      </c>
-      <c r="E9">
-        <v>5.9999999909110224</v>
-      </c>
-      <c r="F9">
-        <v>8.1029430921547796</v>
-      </c>
-      <c r="G9">
-        <v>4.7263752422845942</v>
-      </c>
-      <c r="H9">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="I9" s="2">
-        <v>0</v>
-      </c>
+      <c r="B9" s="5" cm="1">
+        <f t="array" ref="B9">INDEX($B$2:$M$13, COLUMN(A8), ROW(A8))</f>
+        <v>0.99980301599999999</v>
+      </c>
+      <c r="C9" s="5" cm="1">
+        <f t="array" ref="C9">INDEX($B$2:$M$13, COLUMN(B8), ROW(B8))</f>
+        <v>-0.52043820617740066</v>
+      </c>
+      <c r="D9" s="5" cm="1">
+        <f t="array" ref="D9">INDEX($B$2:$M$13, COLUMN(C8), ROW(C8))</f>
+        <v>1.5040514489777961E-2</v>
+      </c>
+      <c r="E9" s="5" cm="1">
+        <f t="array" ref="E9">INDEX($B$2:$M$13, COLUMN(D8), ROW(D8))</f>
+        <v>-0.45611882530944092</v>
+      </c>
+      <c r="F9" s="5" cm="1">
+        <f t="array" ref="F9">INDEX($B$2:$M$13, COLUMN(E8), ROW(E8))</f>
+        <v>-0.52188075027265435</v>
+      </c>
+      <c r="G9" s="5" cm="1">
+        <f t="array" ref="G9">INDEX($B$2:$M$13, COLUMN(F8), ROW(F8))</f>
+        <v>0.95414290742954877</v>
+      </c>
+      <c r="H9" s="5" cm="1">
+        <f t="array" ref="H9">INDEX($B$2:$M$13, COLUMN(G8), ROW(G8))</f>
+        <v>-0.48652674699673709</v>
+      </c>
+      <c r="I9" s="2"/>
       <c r="J9">
-        <v>32.677864608886978</v>
-      </c>
-      <c r="K9" s="22">
-        <v>1.9463849242714379</v>
+        <v>-0.49633697816267242</v>
+      </c>
+      <c r="K9">
+        <v>-7.2776683015054466E-3</v>
       </c>
       <c r="L9">
-        <v>5.9999999909110224</v>
+        <v>-0.45611882530944092</v>
       </c>
       <c r="M9">
-        <v>25.116701684381109</v>
+        <v>-0.51582475030189401</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="18">
+      <c r="A10">
         <v>8</v>
       </c>
-      <c r="B10" s="5">
-        <v>31.369988580000001</v>
-      </c>
-      <c r="C10" s="22">
-        <v>0.43360638701186949</v>
-      </c>
-      <c r="D10">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="E10">
-        <v>5.9999999909110224</v>
-      </c>
-      <c r="F10">
-        <v>4.9907655103560211</v>
-      </c>
-      <c r="G10">
-        <v>23.876910448498951</v>
-      </c>
-      <c r="H10" s="22">
-        <v>2.2720076497793468E-2</v>
-      </c>
-      <c r="I10">
-        <v>31.873130872286779</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
+      <c r="B10" s="5" cm="1">
+        <f t="array" ref="B10">INDEX($B$2:$M$13, COLUMN(A9), ROW(A9))</f>
+        <v>-0.51208986300000003</v>
+      </c>
+      <c r="C10" s="5" cm="1">
+        <f t="array" ref="C10">INDEX($B$2:$M$13, COLUMN(B9), ROW(B9))</f>
+        <v>0.99958808090207341</v>
+      </c>
+      <c r="D10" s="5" cm="1">
+        <f t="array" ref="D10">INDEX($B$2:$M$13, COLUMN(C9), ROW(C9))</f>
+        <v>-0.34758995247793623</v>
+      </c>
+      <c r="E10" s="5" cm="1">
+        <f t="array" ref="E10">INDEX($B$2:$M$13, COLUMN(D9), ROW(D9))</f>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="F10" s="5" cm="1">
+        <f t="array" ref="F10">INDEX($B$2:$M$13, COLUMN(E9), ROW(E9))</f>
+        <v>-0.22224793613700761</v>
+      </c>
+      <c r="G10" s="5" cm="1">
+        <f t="array" ref="G10">INDEX($B$2:$M$13, COLUMN(F9), ROW(F9))</f>
+        <v>-0.27910231237535182</v>
+      </c>
+      <c r="H10" s="5" cm="1">
+        <f t="array" ref="H10">INDEX($B$2:$M$13, COLUMN(G9), ROW(G9))</f>
+        <v>0.99988684582707787</v>
+      </c>
+      <c r="I10" s="5" cm="1">
+        <f t="array" ref="I10">INDEX($B$2:$M$13, COLUMN(H9), ROW(H9))</f>
+        <v>-0.49633697816267242</v>
+      </c>
+      <c r="J10" s="2"/>
       <c r="K10">
-        <v>32.677864608886978</v>
+        <v>-0.34725050916496952</v>
       </c>
       <c r="L10">
-        <v>5.9999999909110224</v>
-      </c>
-      <c r="M10">
-        <v>7.0176037388854144</v>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="M10" s="12">
+        <v>0.94962382237510101</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11" s="18">
+      <c r="A11">
         <v>9</v>
       </c>
-      <c r="B11" s="5">
-        <v>23.070848359999999</v>
-      </c>
-      <c r="C11">
-        <v>31.03668594136634</v>
-      </c>
-      <c r="D11" s="22">
-        <v>0.42530126497041992</v>
-      </c>
-      <c r="E11">
-        <v>5.9999999909110224</v>
-      </c>
-      <c r="F11">
-        <v>8.1029430921547796</v>
-      </c>
-      <c r="G11">
-        <v>23.876910448498951</v>
-      </c>
-      <c r="H11">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="I11">
-        <v>23.573990654156749</v>
-      </c>
-      <c r="J11">
-        <v>32.677864608886978</v>
-      </c>
-      <c r="K11" s="2">
-        <v>0</v>
-      </c>
+      <c r="B11" s="5" cm="1">
+        <f t="array" ref="B11">INDEX($B$2:$M$13, COLUMN(A10), ROW(A10))</f>
+        <v>-7.01493E-3</v>
+      </c>
+      <c r="C11" s="5" cm="1">
+        <f t="array" ref="C11">INDEX($B$2:$M$13, COLUMN(B10), ROW(B10))</f>
+        <v>-0.34708422671409428</v>
+      </c>
+      <c r="D11" s="5" cm="1">
+        <f t="array" ref="D11">INDEX($B$2:$M$13, COLUMN(C10), ROW(C10))</f>
+        <v>0.99966055668703313</v>
+      </c>
+      <c r="E11" s="5" cm="1">
+        <f t="array" ref="E11">INDEX($B$2:$M$13, COLUMN(D10), ROW(D10))</f>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="F11" s="5" cm="1">
+        <f t="array" ref="F11">INDEX($B$2:$M$13, COLUMN(E10), ROW(E10))</f>
+        <v>-0.36512160936794091</v>
+      </c>
+      <c r="G11" s="5" cm="1">
+        <f t="array" ref="G11">INDEX($B$2:$M$13, COLUMN(F10), ROW(F10))</f>
+        <v>-0.27910231237535171</v>
+      </c>
+      <c r="H11" s="5" cm="1">
+        <f t="array" ref="H11">INDEX($B$2:$M$13, COLUMN(G10), ROW(G10))</f>
+        <v>-0.34038701134538812</v>
+      </c>
+      <c r="I11" s="5" cm="1">
+        <f t="array" ref="I11">INDEX($B$2:$M$13, COLUMN(H10), ROW(H10))</f>
+        <v>-7.2776683015054466E-3</v>
+      </c>
+      <c r="J11" s="5" cm="1">
+        <f t="array" ref="J11">INDEX($B$2:$M$13, COLUMN(I10), ROW(I10))</f>
+        <v>-0.34725050916496952</v>
+      </c>
+      <c r="K11" s="2"/>
       <c r="L11">
-        <v>5.9999999909110224</v>
+        <v>-0.31911282313630129</v>
       </c>
       <c r="M11">
-        <v>24.65327670241172</v>
+        <v>-3.6364654371126022E-2</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12" s="18">
+      <c r="A12">
         <v>10</v>
       </c>
-      <c r="B12" s="5">
-        <v>31.182488580000001</v>
-      </c>
-      <c r="C12">
-        <v>31.274132205425509</v>
-      </c>
-      <c r="D12">
-        <v>33.1031658738574</v>
-      </c>
-      <c r="E12" s="22">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>2.6654431003916672</v>
-      </c>
-      <c r="G12">
-        <v>28.50137308568231</v>
-      </c>
-      <c r="H12">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="I12">
-        <v>31.779380872428789</v>
-      </c>
-      <c r="J12">
-        <v>32.584114609028987</v>
-      </c>
-      <c r="K12">
-        <v>32.584114609028987</v>
-      </c>
-      <c r="L12" s="2">
-        <v>0</v>
-      </c>
+      <c r="B12" s="5" cm="1">
+        <f t="array" ref="B12">INDEX($B$2:$M$13, COLUMN(A11), ROW(A11))</f>
+        <v>-0.43965200500000001</v>
+      </c>
+      <c r="C12" s="5" cm="1">
+        <f t="array" ref="C12">INDEX($B$2:$M$13, COLUMN(B11), ROW(B11))</f>
+        <v>-0.29518783809240762</v>
+      </c>
+      <c r="D12" s="5" cm="1">
+        <f t="array" ref="D12">INDEX($B$2:$M$13, COLUMN(C11), ROW(C11))</f>
+        <v>-0.34038701134538812</v>
+      </c>
+      <c r="E12" s="5" cm="1">
+        <f t="array" ref="E12">INDEX($B$2:$M$13, COLUMN(D11), ROW(D11))</f>
+        <v>0.99999999999999944</v>
+      </c>
+      <c r="F12" s="5" cm="1">
+        <f t="array" ref="F12">INDEX($B$2:$M$13, COLUMN(E11), ROW(E11))</f>
+        <v>0.99493667632618188</v>
+      </c>
+      <c r="G12" s="5" cm="1">
+        <f t="array" ref="G12">INDEX($B$2:$M$13, COLUMN(F11), ROW(F11))</f>
+        <v>-0.45083481733371611</v>
+      </c>
+      <c r="H12" s="5" cm="1">
+        <f t="array" ref="H12">INDEX($B$2:$M$13, COLUMN(G11), ROW(G11))</f>
+        <v>-0.33333333333333331</v>
+      </c>
+      <c r="I12" s="5" cm="1">
+        <f t="array" ref="I12">INDEX($B$2:$M$13, COLUMN(H11), ROW(H11))</f>
+        <v>-0.45611882530944092</v>
+      </c>
+      <c r="J12" s="5" cm="1">
+        <f t="array" ref="J12">INDEX($B$2:$M$13, COLUMN(I11), ROW(I11))</f>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="K12" s="5" cm="1">
+        <f t="array" ref="K12">INDEX($B$2:$M$13, COLUMN(J11), ROW(J11))</f>
+        <v>-0.31911282313630129</v>
+      </c>
+      <c r="L12" s="2"/>
       <c r="M12">
-        <v>32.433720656908612</v>
+        <v>-0.46159181056844312</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A13" s="18">
+      <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13" s="5">
-        <v>24.43904822</v>
-      </c>
-      <c r="C13" s="22">
-        <v>1.5630732009148851</v>
-      </c>
-      <c r="D13">
-        <v>2.4633407591518521</v>
-      </c>
-      <c r="E13">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="F13">
-        <v>29.692229823578771</v>
-      </c>
-      <c r="G13">
-        <v>21.621905309297279</v>
-      </c>
-      <c r="H13">
-        <v>0.38529015584062748</v>
-      </c>
-      <c r="I13">
-        <v>24.516889250982771</v>
-      </c>
-      <c r="J13">
-        <v>0.78220618682352216</v>
-      </c>
-      <c r="K13">
-        <v>2.4633407591518521</v>
-      </c>
-      <c r="L13">
-        <v>33.219280949017893</v>
-      </c>
-      <c r="M13" s="2">
-        <v>0</v>
-      </c>
+      <c r="B13" s="5" cm="1">
+        <f t="array" ref="B13">INDEX($B$2:$M$13, COLUMN(A12), ROW(A12))</f>
+        <v>-0.53271688299999997</v>
+      </c>
+      <c r="C13" s="5" cm="1">
+        <f t="array" ref="C13">INDEX($B$2:$M$13, COLUMN(B12), ROW(B12))</f>
+        <v>0.94871716359144431</v>
+      </c>
+      <c r="D13" s="5" cm="1">
+        <f t="array" ref="D13">INDEX($B$2:$M$13, COLUMN(C12), ROW(C12))</f>
+        <v>-3.6364654371126022E-2</v>
+      </c>
+      <c r="E13" s="5" cm="1">
+        <f t="array" ref="E13">INDEX($B$2:$M$13, COLUMN(D12), ROW(D12))</f>
+        <v>-0.46159181056844312</v>
+      </c>
+      <c r="F13" s="5" cm="1">
+        <f t="array" ref="F13">INDEX($B$2:$M$13, COLUMN(E12), ROW(E12))</f>
+        <v>-0.37416950215763012</v>
+      </c>
+      <c r="G13" s="5" cm="1">
+        <f t="array" ref="G13">INDEX($B$2:$M$13, COLUMN(F12), ROW(F12))</f>
+        <v>-0.37458298728065398</v>
+      </c>
+      <c r="H13" s="5" cm="1">
+        <f t="array" ref="H13">INDEX($B$2:$M$13, COLUMN(G12), ROW(G12))</f>
+        <v>0.95203310929741403</v>
+      </c>
+      <c r="I13" s="5" cm="1">
+        <f t="array" ref="I13">INDEX($B$2:$M$13, COLUMN(H12), ROW(H12))</f>
+        <v>-0.51582475030189401</v>
+      </c>
+      <c r="J13" s="5" cm="1">
+        <f t="array" ref="J13">INDEX($B$2:$M$13, COLUMN(I12), ROW(I12))</f>
+        <v>0.94962382237510101</v>
+      </c>
+      <c r="K13" s="5" cm="1">
+        <f t="array" ref="K13">INDEX($B$2:$M$13, COLUMN(J12), ROW(J12))</f>
+        <v>-3.6364654371126022E-2</v>
+      </c>
+      <c r="L13" s="5" cm="1">
+        <f t="array" ref="L13">INDEX($B$2:$M$13, COLUMN(K12), ROW(K12))</f>
+        <v>-0.46159181056844312</v>
+      </c>
+      <c r="M13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3A708D-B166-5745-9C6D-152DDC697D75}">
   <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4193,28 +4871,28 @@
       <c r="E2">
         <v>0.898984279</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2">
         <v>0.90116766699999995</v>
       </c>
-      <c r="G2" s="14">
+      <c r="G2" s="12">
         <v>0.10209418000000001</v>
       </c>
-      <c r="H2" s="12">
+      <c r="H2">
         <v>0.99999999399999995</v>
       </c>
-      <c r="I2" s="14">
+      <c r="I2" s="12">
         <v>1.97554E-3</v>
       </c>
-      <c r="J2" s="12">
+      <c r="J2">
         <v>0.97847743700000001</v>
       </c>
-      <c r="K2" s="12">
+      <c r="K2">
         <v>0.52980522200000002</v>
       </c>
       <c r="L2">
         <v>0.898984279</v>
       </c>
-      <c r="M2" s="23">
+      <c r="M2" s="10">
         <v>0.75799431799999994</v>
       </c>
       <c r="O2" s="3" t="s">
@@ -4263,13 +4941,13 @@
       <c r="G3">
         <v>0.57409199933194033</v>
       </c>
-      <c r="H3" s="14">
+      <c r="H3" s="12">
         <v>3.1977288258686877E-2</v>
       </c>
       <c r="I3">
         <v>0.93178139663832171</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="12">
         <v>1.4122453821440881E-2</v>
       </c>
       <c r="K3">
@@ -4278,7 +4956,7 @@
       <c r="L3">
         <v>0.86192899489150898</v>
       </c>
-      <c r="M3" s="14">
+      <c r="M3" s="12">
         <v>0.1125428549791273</v>
       </c>
       <c r="O3" s="3" t="s">
@@ -4337,7 +5015,7 @@
       <c r="J4">
         <v>0.99999999406987683</v>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="12">
         <v>1.56249973338024E-2</v>
       </c>
       <c r="L4">
@@ -4388,7 +5066,7 @@
         <v>0.99999999540183959</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="14">
+      <c r="F5" s="12">
         <v>4.85386120900336E-2</v>
       </c>
       <c r="G5">
@@ -4406,7 +5084,7 @@
       <c r="K5">
         <v>0.94176634311228846</v>
       </c>
-      <c r="L5" s="14">
+      <c r="L5" s="12">
         <v>0</v>
       </c>
       <c r="M5">
@@ -4473,7 +5151,7 @@
       <c r="K6">
         <v>0.94286685456228247</v>
       </c>
-      <c r="L6" s="14">
+      <c r="L6" s="12">
         <v>4.85386120900336E-2</v>
       </c>
       <c r="M6">
@@ -4548,23 +5226,23 @@
         <f t="array" ref="B8">INDEX($B$2:$M$13, COLUMN(A7), ROW(A7))</f>
         <v>0.99999999399999995</v>
       </c>
-      <c r="C8" s="13" cm="1">
+      <c r="C8" s="5" cm="1">
         <f t="array" ref="C8">INDEX($B$2:$M$13, COLUMN(B7), ROW(B7))</f>
         <v>3.1977288258686877E-2</v>
       </c>
-      <c r="D8" s="13" cm="1">
+      <c r="D8" s="5" cm="1">
         <f t="array" ref="D8">INDEX($B$2:$M$13, COLUMN(C7), ROW(C7))</f>
         <v>0.99999999540183959</v>
       </c>
-      <c r="E8" s="13" cm="1">
+      <c r="E8" s="5" cm="1">
         <f t="array" ref="E8">INDEX($B$2:$M$13, COLUMN(D7), ROW(D7))</f>
         <v>0.99999999673380247</v>
       </c>
-      <c r="F8" s="13" cm="1">
+      <c r="F8" s="5" cm="1">
         <f t="array" ref="F8">INDEX($B$2:$M$13, COLUMN(E7), ROW(E7))</f>
         <v>0.76921846561984752</v>
       </c>
-      <c r="G8" s="13" cm="1">
+      <c r="G8" s="5" cm="1">
         <f t="array" ref="G8">INDEX($B$2:$M$13, COLUMN(F7), ROW(F7))</f>
         <v>0.66968540079695238</v>
       </c>
@@ -4572,7 +5250,7 @@
       <c r="I8">
         <v>0.99999999388987537</v>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="12">
         <v>7.8568733577535563E-3</v>
       </c>
       <c r="K8">
@@ -4581,7 +5259,7 @@
       <c r="L8">
         <v>0.99999999673380247</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="12">
         <v>0.12844187041346949</v>
       </c>
     </row>
@@ -4593,23 +5271,23 @@
         <f t="array" ref="B9">INDEX($B$2:$M$13, COLUMN(A8), ROW(A8))</f>
         <v>1.97554E-3</v>
       </c>
-      <c r="C9" s="13" cm="1">
+      <c r="C9" s="5" cm="1">
         <f t="array" ref="C9">INDEX($B$2:$M$13, COLUMN(B8), ROW(B8))</f>
         <v>0.93178139663832171</v>
       </c>
-      <c r="D9" s="13" cm="1">
+      <c r="D9" s="5" cm="1">
         <f t="array" ref="D9">INDEX($B$2:$M$13, COLUMN(C8), ROW(C8))</f>
         <v>0.49654243649162871</v>
       </c>
-      <c r="E9" s="13" cm="1">
+      <c r="E9" s="5" cm="1">
         <f t="array" ref="E9">INDEX($B$2:$M$13, COLUMN(D8), ROW(D8))</f>
         <v>0.94176634160032413</v>
       </c>
-      <c r="F9" s="13" cm="1">
+      <c r="F9" s="5" cm="1">
         <f t="array" ref="F9">INDEX($B$2:$M$13, COLUMN(E8), ROW(E8))</f>
         <v>0.94286685305031814</v>
       </c>
-      <c r="G9" s="13" cm="1">
+      <c r="G9" s="5" cm="1">
         <f t="array" ref="G9">INDEX($B$2:$M$13, COLUMN(F8), ROW(F8))</f>
         <v>0.1137096140315057</v>
       </c>
@@ -4639,23 +5317,23 @@
         <f t="array" ref="B10">INDEX($B$2:$M$13, COLUMN(A9), ROW(A9))</f>
         <v>0.97847743700000001</v>
       </c>
-      <c r="C10" s="13" cm="1">
+      <c r="C10" s="5" cm="1">
         <f t="array" ref="C10">INDEX($B$2:$M$13, COLUMN(B9), ROW(B9))</f>
         <v>1.4122453821440881E-2</v>
       </c>
-      <c r="D10" s="13" cm="1">
+      <c r="D10" s="5" cm="1">
         <f t="array" ref="D10">INDEX($B$2:$M$13, COLUMN(C9), ROW(C9))</f>
         <v>0.99999999406987683</v>
       </c>
-      <c r="E10" s="13" cm="1">
+      <c r="E10" s="5" cm="1">
         <f t="array" ref="E10">INDEX($B$2:$M$13, COLUMN(D9), ROW(D9))</f>
         <v>0.94176634311228846</v>
       </c>
-      <c r="F10" s="13" cm="1">
+      <c r="F10" s="5" cm="1">
         <f t="array" ref="F10">INDEX($B$2:$M$13, COLUMN(E9), ROW(E9))</f>
         <v>0.71310297216078933</v>
       </c>
-      <c r="G10" s="13" cm="1">
+      <c r="G10" s="5" cm="1">
         <f t="array" ref="G10">INDEX($B$2:$M$13, COLUMN(F9), ROW(F9))</f>
         <v>0.63897666774550965</v>
       </c>
@@ -4674,7 +5352,7 @@
       <c r="L10">
         <v>0.94176634311228846</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="12">
         <v>0.13488801488488661</v>
       </c>
     </row>
@@ -4686,23 +5364,23 @@
         <f t="array" ref="B11">INDEX($B$2:$M$13, COLUMN(A10), ROW(A10))</f>
         <v>0.52980522200000002</v>
       </c>
-      <c r="C11" s="13" cm="1">
+      <c r="C11" s="5" cm="1">
         <f t="array" ref="C11">INDEX($B$2:$M$13, COLUMN(B10), ROW(B10))</f>
         <v>0.91659001910793603</v>
       </c>
-      <c r="D11" s="13" cm="1">
+      <c r="D11" s="5" cm="1">
         <f t="array" ref="D11">INDEX($B$2:$M$13, COLUMN(C10), ROW(C10))</f>
         <v>1.56249973338024E-2</v>
       </c>
-      <c r="E11" s="13" cm="1">
+      <c r="E11" s="5" cm="1">
         <f t="array" ref="E11">INDEX($B$2:$M$13, COLUMN(D10), ROW(D10))</f>
         <v>0.94176634311228846</v>
       </c>
-      <c r="F11" s="13" cm="1">
+      <c r="F11" s="5" cm="1">
         <f t="array" ref="F11">INDEX($B$2:$M$13, COLUMN(E10), ROW(E10))</f>
         <v>0.94286685456228247</v>
       </c>
-      <c r="G11" s="13" cm="1">
+      <c r="G11" s="5" cm="1">
         <f t="array" ref="G11">INDEX($B$2:$M$13, COLUMN(F10), ROW(F10))</f>
         <v>0.63897666774550965</v>
       </c>
@@ -4734,23 +5412,23 @@
         <f t="array" ref="B12">INDEX($B$2:$M$13, COLUMN(A11), ROW(A11))</f>
         <v>0.898984279</v>
       </c>
-      <c r="C12" s="13" cm="1">
+      <c r="C12" s="5" cm="1">
         <f t="array" ref="C12">INDEX($B$2:$M$13, COLUMN(B11), ROW(B11))</f>
         <v>0.86192899489150898</v>
       </c>
-      <c r="D12" s="13" cm="1">
+      <c r="D12" s="5" cm="1">
         <f t="array" ref="D12">INDEX($B$2:$M$13, COLUMN(C11), ROW(C11))</f>
         <v>0.99999999540183959</v>
       </c>
-      <c r="E12" s="13" cm="1">
+      <c r="E12" s="5" cm="1">
         <f t="array" ref="E12">INDEX($B$2:$M$13, COLUMN(D11), ROW(D11))</f>
         <v>0</v>
       </c>
-      <c r="F12" s="13" cm="1">
+      <c r="F12" s="5" cm="1">
         <f t="array" ref="F12">INDEX($B$2:$M$13, COLUMN(E11), ROW(E11))</f>
         <v>4.85386120900336E-2</v>
       </c>
-      <c r="G12" s="13" cm="1">
+      <c r="G12" s="5" cm="1">
         <f t="array" ref="G12">INDEX($B$2:$M$13, COLUMN(F11), ROW(F11))</f>
         <v>0.76921846265195981</v>
       </c>
@@ -4783,23 +5461,23 @@
         <f t="array" ref="B13">INDEX($B$2:$M$13, COLUMN(A12), ROW(A12))</f>
         <v>0.75799431799999994</v>
       </c>
-      <c r="C13" s="13" cm="1">
+      <c r="C13" s="5" cm="1">
         <f t="array" ref="C13">INDEX($B$2:$M$13, COLUMN(B12), ROW(B12))</f>
         <v>0.1125428549791273</v>
       </c>
-      <c r="D13" s="13" cm="1">
+      <c r="D13" s="5" cm="1">
         <f t="array" ref="D13">INDEX($B$2:$M$13, COLUMN(C12), ROW(C12))</f>
         <v>0.56961422392004091</v>
       </c>
-      <c r="E13" s="13" cm="1">
+      <c r="E13" s="5" cm="1">
         <f t="array" ref="E13">INDEX($B$2:$M$13, COLUMN(D12), ROW(D12))</f>
         <v>0.99999999522462346</v>
       </c>
-      <c r="F13" s="13" cm="1">
+      <c r="F13" s="5" cm="1">
         <f t="array" ref="F13">INDEX($B$2:$M$13, COLUMN(E12), ROW(E12))</f>
         <v>0.78637322429393663</v>
       </c>
-      <c r="G13" s="13" cm="1">
+      <c r="G13" s="5" cm="1">
         <f t="array" ref="G13">INDEX($B$2:$M$13, COLUMN(F12), ROW(F12))</f>
         <v>0.50773717296655807</v>
       </c>
@@ -4826,673 +5504,10 @@
       <c r="M13" s="2"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A16" s="16"/>
+      <c r="A16" s="14"/>
     </row>
     <row r="17" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D17" s="5"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3125F5A-7234-5647-851D-0D6A6A07A661}">
-  <dimension ref="A1:T13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="10.33203125" customWidth="1"/>
-    <col min="2" max="9" width="5.5" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" customWidth="1"/>
-    <col min="11" max="11" width="8.1640625" customWidth="1"/>
-    <col min="12" max="12" width="7.5" customWidth="1"/>
-    <col min="13" max="13" width="6.1640625" customWidth="1"/>
-    <col min="15" max="15" width="4.1640625" customWidth="1"/>
-    <col min="16" max="16" width="11" customWidth="1"/>
-    <col min="17" max="17" width="9.6640625" customWidth="1"/>
-    <col min="18" max="18" width="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.1640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="1">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1">
-        <v>11</v>
-      </c>
-      <c r="P1" s="9">
-        <v>3</v>
-      </c>
-      <c r="Q1" s="9">
-        <v>9</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="S1" s="6"/>
-      <c r="T1" s="7"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="5">
-        <v>-0.53587699799999999</v>
-      </c>
-      <c r="D2">
-        <v>1.5031991999999999E-2</v>
-      </c>
-      <c r="E2">
-        <v>-0.43965200500000001</v>
-      </c>
-      <c r="F2">
-        <v>-0.50661061399999996</v>
-      </c>
-      <c r="G2" s="14">
-        <v>0.95141007099999997</v>
-      </c>
-      <c r="H2">
-        <v>-0.50245943400000004</v>
-      </c>
-      <c r="I2" s="24">
-        <v>0.99980301599999999</v>
-      </c>
-      <c r="J2">
-        <v>-0.51208986300000003</v>
-      </c>
-      <c r="K2">
-        <v>-7.01493E-3</v>
-      </c>
-      <c r="L2">
-        <v>-0.43965200500000001</v>
-      </c>
-      <c r="M2" s="10">
-        <v>-0.53271688299999997</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="P2" cm="1">
-        <f t="array" ref="P2">INDEX(PPM!$B$2:$M$5, ROW(A1), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1.0000000001</v>
-      </c>
-      <c r="Q2" cm="1">
-        <f t="array" ref="Q2">INDEX(PPM!$B$2:$M$5, ROW(B1), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1.5625000100000001E-2</v>
-      </c>
-      <c r="R2" s="5"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" cm="1">
-        <f t="array" ref="B3">INDEX($B$2:$M$13, COLUMN(A2), ROW(A2))</f>
-        <v>-0.53587699799999999</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3">
-        <v>-0.3481711293029694</v>
-      </c>
-      <c r="E3">
-        <v>-0.29518783809240762</v>
-      </c>
-      <c r="F3">
-        <v>-0.19767811977548069</v>
-      </c>
-      <c r="G3">
-        <v>-0.30403879734200751</v>
-      </c>
-      <c r="H3" s="14">
-        <v>0.99909729815891835</v>
-      </c>
-      <c r="I3">
-        <v>-0.52043820617740066</v>
-      </c>
-      <c r="J3" s="14">
-        <v>0.99958808090207341</v>
-      </c>
-      <c r="K3">
-        <v>-0.34708422671409428</v>
-      </c>
-      <c r="L3">
-        <v>-0.29518783809240762</v>
-      </c>
-      <c r="M3" s="14">
-        <v>0.94871716359144431</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="P3" cm="1">
-        <f t="array" ref="P3">INDEX(PPM!$B$2:$M$5, ROW(A2), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1E-10</v>
-      </c>
-      <c r="Q3" cm="1">
-        <f t="array" ref="Q3">INDEX(PPM!$B$2:$M$5, ROW(B2), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>0.98437500010000001</v>
-      </c>
-      <c r="R3" s="5"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" s="5" cm="1">
-        <f t="array" ref="B4">INDEX($B$2:$M$13, COLUMN(A3), ROW(A3))</f>
-        <v>1.5031991999999999E-2</v>
-      </c>
-      <c r="C4" s="5" cm="1">
-        <f t="array" ref="C4">INDEX($B$2:$M$13, COLUMN(B3), ROW(B3))</f>
-        <v>-0.3481711293029694</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4">
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="F4">
-        <v>-0.38704402483723771</v>
-      </c>
-      <c r="G4">
-        <v>-0.25608356496295148</v>
-      </c>
-      <c r="H4">
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="I4">
-        <v>1.5040514489777961E-2</v>
-      </c>
-      <c r="J4">
-        <v>-0.34758995247793623</v>
-      </c>
-      <c r="K4" s="14">
-        <v>0.99966055668703313</v>
-      </c>
-      <c r="L4">
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="M4">
-        <v>-3.6364654371126022E-2</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="P4" cm="1">
-        <f t="array" ref="P4">INDEX(PPM!$B$2:$M$5, ROW(A3), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1E-10</v>
-      </c>
-      <c r="Q4" cm="1">
-        <f t="array" ref="Q4">INDEX(PPM!$B$2:$M$5, ROW(B3), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1E-10</v>
-      </c>
-      <c r="R4" s="5"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" cm="1">
-        <f t="array" ref="B5">INDEX($B$2:$M$13, COLUMN(A4), ROW(A4))</f>
-        <v>-0.43965200500000001</v>
-      </c>
-      <c r="C5" s="5" cm="1">
-        <f t="array" ref="C5">INDEX($B$2:$M$13, COLUMN(B4), ROW(B4))</f>
-        <v>-0.29518783809240762</v>
-      </c>
-      <c r="D5" s="5" cm="1">
-        <f t="array" ref="D5">INDEX($B$2:$M$13, COLUMN(C4), ROW(C4))</f>
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="14">
-        <v>0.99493667632618188</v>
-      </c>
-      <c r="G5">
-        <v>-0.45083481733371611</v>
-      </c>
-      <c r="H5">
-        <v>-0.33333333333333331</v>
-      </c>
-      <c r="I5">
-        <v>-0.45611882530944092</v>
-      </c>
-      <c r="J5">
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="K5">
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="L5" s="14">
-        <v>0.99999999999999944</v>
-      </c>
-      <c r="M5">
-        <v>-0.46159181056844312</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="P5" cm="1">
-        <f t="array" ref="P5">INDEX(PPM!$B$2:$M$5, ROW(A4), MATCH(P$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1E-10</v>
-      </c>
-      <c r="Q5" cm="1">
-        <f t="array" ref="Q5">INDEX(PPM!$B$2:$M$5, ROW(B4), MATCH(Q$1, PPM!$B$1:$M$1, 0)) + 0.0000000001</f>
-        <v>1E-10</v>
-      </c>
-      <c r="R5" s="5"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" s="5" cm="1">
-        <f t="array" ref="B6">INDEX($B$2:$M$13, COLUMN(A5), ROW(A5))</f>
-        <v>-0.50661061399999996</v>
-      </c>
-      <c r="C6" s="5" cm="1">
-        <f t="array" ref="C6">INDEX($B$2:$M$13, COLUMN(B5), ROW(B5))</f>
-        <v>-0.19767811977548069</v>
-      </c>
-      <c r="D6" s="5" cm="1">
-        <f t="array" ref="D6">INDEX($B$2:$M$13, COLUMN(C5), ROW(C5))</f>
-        <v>-0.38704402483723771</v>
-      </c>
-      <c r="E6" s="5" cm="1">
-        <f t="array" ref="E6">INDEX($B$2:$M$13, COLUMN(D5), ROW(D5))</f>
-        <v>0.99493667632618188</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6">
-        <v>-0.49340730420314183</v>
-      </c>
-      <c r="H6">
-        <v>-0.23688968483956721</v>
-      </c>
-      <c r="I6">
-        <v>-0.52188075027265435</v>
-      </c>
-      <c r="J6">
-        <v>-0.22224793613700761</v>
-      </c>
-      <c r="K6">
-        <v>-0.36512160936794091</v>
-      </c>
-      <c r="L6" s="14">
-        <v>0.99493667632618188</v>
-      </c>
-      <c r="M6">
-        <v>-0.37416950215763012</v>
-      </c>
-      <c r="R6">
-        <f>CORREL(P2:P5, Q2:Q5)</f>
-        <v>-0.3191128231363014</v>
-      </c>
-      <c r="S6" s="3"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" cm="1">
-        <f t="array" ref="B7">INDEX($B$2:$M$13, COLUMN(A6), ROW(A6))</f>
-        <v>0.95141007099999997</v>
-      </c>
-      <c r="C7" s="5" cm="1">
-        <f t="array" ref="C7">INDEX($B$2:$M$13, COLUMN(B6), ROW(B6))</f>
-        <v>-0.30403879734200751</v>
-      </c>
-      <c r="D7" s="5" cm="1">
-        <f t="array" ref="D7">INDEX($B$2:$M$13, COLUMN(C6), ROW(C6))</f>
-        <v>-0.25608356496295148</v>
-      </c>
-      <c r="E7" s="5" cm="1">
-        <f t="array" ref="E7">INDEX($B$2:$M$13, COLUMN(D6), ROW(D6))</f>
-        <v>-0.45083481733371611</v>
-      </c>
-      <c r="F7" s="5" cm="1">
-        <f t="array" ref="F7">INDEX($B$2:$M$13, COLUMN(E6), ROW(E6))</f>
-        <v>-0.49340730420314183</v>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7">
-        <v>-0.27050089040022968</v>
-      </c>
-      <c r="I7" s="14">
-        <v>0.95414290742954877</v>
-      </c>
-      <c r="J7">
-        <v>-0.27910231237535182</v>
-      </c>
-      <c r="K7">
-        <v>-0.27910231237535171</v>
-      </c>
-      <c r="L7">
-        <v>-0.45083481733371611</v>
-      </c>
-      <c r="M7">
-        <v>-0.37458298728065398</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" cm="1">
-        <f t="array" ref="B8">INDEX($B$2:$M$13, COLUMN(A7), ROW(A7))</f>
-        <v>-0.50245943400000004</v>
-      </c>
-      <c r="C8" s="5" cm="1">
-        <f t="array" ref="C8">INDEX($B$2:$M$13, COLUMN(B7), ROW(B7))</f>
-        <v>0.99909729815891835</v>
-      </c>
-      <c r="D8" s="5" cm="1">
-        <f t="array" ref="D8">INDEX($B$2:$M$13, COLUMN(C7), ROW(C7))</f>
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="E8" s="5" cm="1">
-        <f t="array" ref="E8">INDEX($B$2:$M$13, COLUMN(D7), ROW(D7))</f>
-        <v>-0.33333333333333331</v>
-      </c>
-      <c r="F8" s="5" cm="1">
-        <f t="array" ref="F8">INDEX($B$2:$M$13, COLUMN(E7), ROW(E7))</f>
-        <v>-0.23688968483956721</v>
-      </c>
-      <c r="G8" s="5" cm="1">
-        <f t="array" ref="G8">INDEX($B$2:$M$13, COLUMN(F7), ROW(F7))</f>
-        <v>-0.27050089040022968</v>
-      </c>
-      <c r="H8" s="2"/>
-      <c r="I8">
-        <v>-0.48652674699673709</v>
-      </c>
-      <c r="J8" s="14">
-        <v>0.99988684582707787</v>
-      </c>
-      <c r="K8">
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="L8">
-        <v>-0.33333333333333331</v>
-      </c>
-      <c r="M8" s="14">
-        <v>0.95203310929741403</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" s="5" cm="1">
-        <f t="array" ref="B9">INDEX($B$2:$M$13, COLUMN(A8), ROW(A8))</f>
-        <v>0.99980301599999999</v>
-      </c>
-      <c r="C9" s="5" cm="1">
-        <f t="array" ref="C9">INDEX($B$2:$M$13, COLUMN(B8), ROW(B8))</f>
-        <v>-0.52043820617740066</v>
-      </c>
-      <c r="D9" s="13" cm="1">
-        <f t="array" ref="D9">INDEX($B$2:$M$13, COLUMN(C8), ROW(C8))</f>
-        <v>1.5040514489777961E-2</v>
-      </c>
-      <c r="E9" s="13" cm="1">
-        <f t="array" ref="E9">INDEX($B$2:$M$13, COLUMN(D8), ROW(D8))</f>
-        <v>-0.45611882530944092</v>
-      </c>
-      <c r="F9" s="13" cm="1">
-        <f t="array" ref="F9">INDEX($B$2:$M$13, COLUMN(E8), ROW(E8))</f>
-        <v>-0.52188075027265435</v>
-      </c>
-      <c r="G9" s="13" cm="1">
-        <f t="array" ref="G9">INDEX($B$2:$M$13, COLUMN(F8), ROW(F8))</f>
-        <v>0.95414290742954877</v>
-      </c>
-      <c r="H9" s="5" cm="1">
-        <f t="array" ref="H9">INDEX($B$2:$M$13, COLUMN(G8), ROW(G8))</f>
-        <v>-0.48652674699673709</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9">
-        <v>-0.49633697816267242</v>
-      </c>
-      <c r="K9">
-        <v>-7.2776683015054466E-3</v>
-      </c>
-      <c r="L9">
-        <v>-0.45611882530944092</v>
-      </c>
-      <c r="M9">
-        <v>-0.51582475030189401</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" s="5" cm="1">
-        <f t="array" ref="B10">INDEX($B$2:$M$13, COLUMN(A9), ROW(A9))</f>
-        <v>-0.51208986300000003</v>
-      </c>
-      <c r="C10" s="5" cm="1">
-        <f t="array" ref="C10">INDEX($B$2:$M$13, COLUMN(B9), ROW(B9))</f>
-        <v>0.99958808090207341</v>
-      </c>
-      <c r="D10" s="13" cm="1">
-        <f t="array" ref="D10">INDEX($B$2:$M$13, COLUMN(C9), ROW(C9))</f>
-        <v>-0.34758995247793623</v>
-      </c>
-      <c r="E10" s="13" cm="1">
-        <f t="array" ref="E10">INDEX($B$2:$M$13, COLUMN(D9), ROW(D9))</f>
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="F10" s="13" cm="1">
-        <f t="array" ref="F10">INDEX($B$2:$M$13, COLUMN(E9), ROW(E9))</f>
-        <v>-0.22224793613700761</v>
-      </c>
-      <c r="G10" s="13" cm="1">
-        <f t="array" ref="G10">INDEX($B$2:$M$13, COLUMN(F9), ROW(F9))</f>
-        <v>-0.27910231237535182</v>
-      </c>
-      <c r="H10" s="5" cm="1">
-        <f t="array" ref="H10">INDEX($B$2:$M$13, COLUMN(G9), ROW(G9))</f>
-        <v>0.99988684582707787</v>
-      </c>
-      <c r="I10" s="5" cm="1">
-        <f t="array" ref="I10">INDEX($B$2:$M$13, COLUMN(H9), ROW(H9))</f>
-        <v>-0.49633697816267242</v>
-      </c>
-      <c r="J10" s="2"/>
-      <c r="K10">
-        <v>-0.34725050916496952</v>
-      </c>
-      <c r="L10">
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="M10" s="14">
-        <v>0.94962382237510101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5" cm="1">
-        <f t="array" ref="B11">INDEX($B$2:$M$13, COLUMN(A10), ROW(A10))</f>
-        <v>-7.01493E-3</v>
-      </c>
-      <c r="C11" s="5" cm="1">
-        <f t="array" ref="C11">INDEX($B$2:$M$13, COLUMN(B10), ROW(B10))</f>
-        <v>-0.34708422671409428</v>
-      </c>
-      <c r="D11" s="13" cm="1">
-        <f t="array" ref="D11">INDEX($B$2:$M$13, COLUMN(C10), ROW(C10))</f>
-        <v>0.99966055668703313</v>
-      </c>
-      <c r="E11" s="13" cm="1">
-        <f t="array" ref="E11">INDEX($B$2:$M$13, COLUMN(D10), ROW(D10))</f>
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="F11" s="13" cm="1">
-        <f t="array" ref="F11">INDEX($B$2:$M$13, COLUMN(E10), ROW(E10))</f>
-        <v>-0.36512160936794091</v>
-      </c>
-      <c r="G11" s="13" cm="1">
-        <f t="array" ref="G11">INDEX($B$2:$M$13, COLUMN(F10), ROW(F10))</f>
-        <v>-0.27910231237535171</v>
-      </c>
-      <c r="H11" s="5" cm="1">
-        <f t="array" ref="H11">INDEX($B$2:$M$13, COLUMN(G10), ROW(G10))</f>
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="I11" s="5" cm="1">
-        <f t="array" ref="I11">INDEX($B$2:$M$13, COLUMN(H10), ROW(H10))</f>
-        <v>-7.2776683015054466E-3</v>
-      </c>
-      <c r="J11" s="5" cm="1">
-        <f t="array" ref="J11">INDEX($B$2:$M$13, COLUMN(I10), ROW(I10))</f>
-        <v>-0.34725050916496952</v>
-      </c>
-      <c r="K11" s="2"/>
-      <c r="L11">
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="M11">
-        <v>-3.6364654371126022E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12" s="5" cm="1">
-        <f t="array" ref="B12">INDEX($B$2:$M$13, COLUMN(A11), ROW(A11))</f>
-        <v>-0.43965200500000001</v>
-      </c>
-      <c r="C12" s="5" cm="1">
-        <f t="array" ref="C12">INDEX($B$2:$M$13, COLUMN(B11), ROW(B11))</f>
-        <v>-0.29518783809240762</v>
-      </c>
-      <c r="D12" s="13" cm="1">
-        <f t="array" ref="D12">INDEX($B$2:$M$13, COLUMN(C11), ROW(C11))</f>
-        <v>-0.34038701134538812</v>
-      </c>
-      <c r="E12" s="13" cm="1">
-        <f t="array" ref="E12">INDEX($B$2:$M$13, COLUMN(D11), ROW(D11))</f>
-        <v>0.99999999999999944</v>
-      </c>
-      <c r="F12" s="13" cm="1">
-        <f t="array" ref="F12">INDEX($B$2:$M$13, COLUMN(E11), ROW(E11))</f>
-        <v>0.99493667632618188</v>
-      </c>
-      <c r="G12" s="13" cm="1">
-        <f t="array" ref="G12">INDEX($B$2:$M$13, COLUMN(F11), ROW(F11))</f>
-        <v>-0.45083481733371611</v>
-      </c>
-      <c r="H12" s="5" cm="1">
-        <f t="array" ref="H12">INDEX($B$2:$M$13, COLUMN(G11), ROW(G11))</f>
-        <v>-0.33333333333333331</v>
-      </c>
-      <c r="I12" s="5" cm="1">
-        <f t="array" ref="I12">INDEX($B$2:$M$13, COLUMN(H11), ROW(H11))</f>
-        <v>-0.45611882530944092</v>
-      </c>
-      <c r="J12" s="5" cm="1">
-        <f t="array" ref="J12">INDEX($B$2:$M$13, COLUMN(I11), ROW(I11))</f>
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="K12" s="5" cm="1">
-        <f t="array" ref="K12">INDEX($B$2:$M$13, COLUMN(J11), ROW(J11))</f>
-        <v>-0.31911282313630129</v>
-      </c>
-      <c r="L12" s="2"/>
-      <c r="M12">
-        <v>-0.46159181056844312</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>11</v>
-      </c>
-      <c r="B13" s="5" cm="1">
-        <f t="array" ref="B13">INDEX($B$2:$M$13, COLUMN(A12), ROW(A12))</f>
-        <v>-0.53271688299999997</v>
-      </c>
-      <c r="C13" s="5" cm="1">
-        <f t="array" ref="C13">INDEX($B$2:$M$13, COLUMN(B12), ROW(B12))</f>
-        <v>0.94871716359144431</v>
-      </c>
-      <c r="D13" s="13" cm="1">
-        <f t="array" ref="D13">INDEX($B$2:$M$13, COLUMN(C12), ROW(C12))</f>
-        <v>-3.6364654371126022E-2</v>
-      </c>
-      <c r="E13" s="13" cm="1">
-        <f t="array" ref="E13">INDEX($B$2:$M$13, COLUMN(D12), ROW(D12))</f>
-        <v>-0.46159181056844312</v>
-      </c>
-      <c r="F13" s="13" cm="1">
-        <f t="array" ref="F13">INDEX($B$2:$M$13, COLUMN(E12), ROW(E12))</f>
-        <v>-0.37416950215763012</v>
-      </c>
-      <c r="G13" s="13" cm="1">
-        <f t="array" ref="G13">INDEX($B$2:$M$13, COLUMN(F12), ROW(F12))</f>
-        <v>-0.37458298728065398</v>
-      </c>
-      <c r="H13" s="5" cm="1">
-        <f t="array" ref="H13">INDEX($B$2:$M$13, COLUMN(G12), ROW(G12))</f>
-        <v>0.95203310929741403</v>
-      </c>
-      <c r="I13" s="5" cm="1">
-        <f t="array" ref="I13">INDEX($B$2:$M$13, COLUMN(H12), ROW(H12))</f>
-        <v>-0.51582475030189401</v>
-      </c>
-      <c r="J13" s="5" cm="1">
-        <f t="array" ref="J13">INDEX($B$2:$M$13, COLUMN(I12), ROW(I12))</f>
-        <v>0.94962382237510101</v>
-      </c>
-      <c r="K13" s="5" cm="1">
-        <f t="array" ref="K13">INDEX($B$2:$M$13, COLUMN(J12), ROW(J12))</f>
-        <v>-3.6364654371126022E-2</v>
-      </c>
-      <c r="L13" s="5" cm="1">
-        <f t="array" ref="L13">INDEX($B$2:$M$13, COLUMN(K12), ROW(K12))</f>
-        <v>-0.46159181056844312</v>
-      </c>
-      <c r="M13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
file cleanup and reverse fasta creation
</commit_message>
<xml_diff>
--- a/ppm_output_handcalc.xlsx
+++ b/ppm_output_handcalc.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/enoch/Documents/Local Erill Research/drirpy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74053477-00C3-F940-8A7A-132A77FD835E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AE05A15-5230-4047-9326-79C288A585AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4520" yWindow="-20940" windowWidth="18960" windowHeight="20800" activeTab="2" xr2:uid="{BF39720B-7314-BE4F-87DC-079655431D8B}"/>
-    <workbookView xWindow="13460" yWindow="-21100" windowWidth="20280" windowHeight="21100" activeTab="3" xr2:uid="{4F083981-888D-6D4A-9A91-0CE6B4D6ABC5}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="2" xr2:uid="{BF39720B-7314-BE4F-87DC-079655431D8B}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" activeTab="3" xr2:uid="{4F083981-888D-6D4A-9A91-0CE6B4D6ABC5}"/>
   </bookViews>
   <sheets>
     <sheet name="PPM" sheetId="1" r:id="rId1"/>
@@ -75,9 +75,6 @@
   </si>
   <si>
     <t>T</t>
-  </si>
-  <si>
-    <t>Metric: Information Content</t>
   </si>
   <si>
     <t>H_after</t>
@@ -183,6 +180,9 @@
   </si>
   <si>
     <t>H_Q</t>
+  </si>
+  <si>
+    <t>Metric: Avg Information Content</t>
   </si>
 </sst>
 </file>
@@ -2614,7 +2614,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="15">
         <v>0</v>
@@ -2659,10 +2659,10 @@
         <v>9</v>
       </c>
       <c r="R1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="S1" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="T1" s="7"/>
     </row>
@@ -3252,7 +3252,7 @@
   <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="9" width="5.5" customWidth="1"/>
     <col min="10" max="10" width="7.83203125" customWidth="1"/>
     <col min="11" max="11" width="8.1640625" customWidth="1"/>
@@ -3269,7 +3269,7 @@
   <sheetData>
     <row r="1" spans="1:22" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -3314,19 +3314,19 @@
         <v>9</v>
       </c>
       <c r="R1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="S1" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="T1" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="V1" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="S1" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="T1" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="U1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="V1" s="7" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.2">
@@ -3994,22 +3994,22 @@
     </row>
     <row r="16" spans="1:22" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
         <v>8</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>9</v>
-      </c>
-      <c r="D16" t="s">
-        <v>10</v>
       </c>
       <c r="L16" s="23"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -4018,13 +4018,13 @@
         <v>9</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L17" s="23"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18">
         <v>1</v>
@@ -4033,12 +4033,12 @@
         <v>6</v>
       </c>
       <c r="D18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -4047,12 +4047,12 @@
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B20">
         <v>3</v>
@@ -4061,12 +4061,12 @@
         <v>4</v>
       </c>
       <c r="D20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21">
         <v>4</v>
@@ -4077,7 +4077,7 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -4088,7 +4088,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23">
         <v>6</v>
@@ -4099,7 +4099,7 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B24">
         <v>7</v>
@@ -4135,7 +4135,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -4180,7 +4180,7 @@
         <v>9</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S1" s="6"/>
       <c r="T1" s="7"/>
@@ -4800,7 +4800,7 @@
   <sheetData>
     <row r="1" spans="1:21" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -4845,16 +4845,16 @@
         <v>7</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="T1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="U1" t="s">
         <v>22</v>
-      </c>
-      <c r="U1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">

</xml_diff>